<commit_message>
Encode Maybe Grandes with ADD attended and LMS setup; clean template rows
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -1528,29 +1528,17 @@
       </c>
       <c r="B9" s="36" t="inlineStr">
         <is>
-          <t>Dela Cruz, Juan M.</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>+63 917 123 4567</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
-        <is>
-          <t>juan.delacruz@gmail.com</t>
-        </is>
-      </c>
-      <c r="E9" s="36" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins (UM)</t>
-        </is>
-      </c>
+          <t>Grandes, Maybe</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr"/>
+      <c r="D9" s="36" t="inlineStr"/>
+      <c r="E9" s="36" t="inlineStr"/>
       <c r="F9" s="37" t="n">
-        <v>46244</v>
+        <v>46279</v>
       </c>
       <c r="G9" s="37" t="n">
-        <v>46249</v>
+        <v>46279</v>
       </c>
       <c r="H9" s="35" t="inlineStr">
         <is>
@@ -1558,30 +1546,28 @@
         </is>
       </c>
       <c r="I9" s="37" t="n">
-        <v>46249</v>
+        <v>46279</v>
       </c>
       <c r="J9" s="36" t="inlineStr">
         <is>
-          <t>Passed initial interview; keen on full-time advisory career</t>
+          <t>Attended ADD on Sept 14; confirmed interest. Preparing for LMS setup.</t>
         </is>
       </c>
       <c r="K9" s="37" t="n">
-        <v>46250</v>
+        <v>46280</v>
       </c>
       <c r="L9" s="35" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M9" s="37" t="n">
-        <v>46259</v>
-      </c>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="M9" s="37" t="n"/>
       <c r="N9" s="38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="36" t="inlineStr">
         <is>
-          <t>Cert #LMS-2026-881 (Passed 94%)</t>
+          <t>Pending account activation</t>
         </is>
       </c>
       <c r="P9" s="35">
@@ -1590,2257 +1576,1529 @@
       </c>
       <c r="Q9" s="36" t="inlineStr">
         <is>
-          <t>Endorse for Insurance Commission Licensing Exam</t>
+          <t>Set up LMS account &amp; send module access link today</t>
         </is>
       </c>
       <c r="R9" s="37" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="S9" s="36" t="inlineStr">
         <is>
-          <t>Submitted all government IDs and 2x2 photo</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Will set up her LMS today.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="39" t="inlineStr">
-        <is>
-          <t>REC-002</t>
-        </is>
-      </c>
-      <c r="B10" s="40" t="inlineStr">
-        <is>
-          <t>Santos, Maria Clara</t>
-        </is>
-      </c>
-      <c r="C10" s="39" t="inlineStr">
-        <is>
-          <t>+63 918 234 5678</t>
-        </is>
-      </c>
-      <c r="D10" s="40" t="inlineStr">
-        <is>
-          <t>maria.santos@yahoo.com</t>
-        </is>
-      </c>
-      <c r="E10" s="40" t="inlineStr">
-        <is>
-          <t>David Tan</t>
-        </is>
-      </c>
-      <c r="F10" s="41" t="n">
-        <v>46246</v>
-      </c>
-      <c r="G10" s="41" t="n">
-        <v>46249</v>
-      </c>
-      <c r="H10" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I10" s="41" t="n">
-        <v>46249</v>
-      </c>
-      <c r="J10" s="40" t="inlineStr">
-        <is>
-          <t>Very active in Q&amp;A session; exploring part-time advisory</t>
-        </is>
-      </c>
-      <c r="K10" s="41" t="n">
-        <v>46251</v>
-      </c>
-      <c r="L10" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M10" s="41" t="n">
-        <v>46262</v>
-      </c>
-      <c r="N10" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="40" t="inlineStr">
-        <is>
-          <t>Cert #LMS-2026-894 (Passed 88%)</t>
-        </is>
-      </c>
+      <c r="A10" s="39">
+        <f>IF(B10="","","REC-"&amp;TEXT(10-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B10" s="40" t="inlineStr"/>
+      <c r="C10" s="39" t="inlineStr"/>
+      <c r="D10" s="40" t="inlineStr"/>
+      <c r="E10" s="40" t="inlineStr"/>
+      <c r="F10" s="41" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="39" t="inlineStr"/>
+      <c r="I10" s="41" t="n"/>
+      <c r="J10" s="40" t="inlineStr"/>
+      <c r="K10" s="41" t="n"/>
+      <c r="L10" s="39" t="inlineStr"/>
+      <c r="M10" s="41" t="n"/>
+      <c r="N10" s="42" t="n"/>
+      <c r="O10" s="40" t="inlineStr"/>
       <c r="P10" s="39">
         <f>IF(B10="","",IF(L10="Yes","LMS Completed (Ready for Exam)",IF(L10="In Progress","LMS In Progress",IF(H10="Yes","ADD Attended - Awaiting LMS",IF(H10="Rescheduled","ADD Rescheduled",IF(H10="Pending","ADD Scheduled",IF(H10="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q10" s="40" t="inlineStr">
-        <is>
-          <t>Review mock exam questions with recruit</t>
-        </is>
-      </c>
-      <c r="R10" s="41" t="n">
-        <v>46282</v>
-      </c>
-      <c r="S10" s="40" t="inlineStr">
-        <is>
-          <t>Exam requirements filed; scheduling mock test</t>
-        </is>
-      </c>
+      <c r="Q10" s="40" t="inlineStr"/>
+      <c r="R10" s="41" t="n"/>
+      <c r="S10" s="40" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>REC-003</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="inlineStr">
-        <is>
-          <t>Reyes, Mark Anthony</t>
-        </is>
-      </c>
-      <c r="C11" s="35" t="inlineStr">
-        <is>
-          <t>+63 919 345 6789</t>
-        </is>
-      </c>
-      <c r="D11" s="36" t="inlineStr">
-        <is>
-          <t>mark.reyes@outlook.com</t>
-        </is>
-      </c>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins (UM)</t>
-        </is>
-      </c>
-      <c r="F11" s="37" t="n">
-        <v>46252</v>
-      </c>
-      <c r="G11" s="37" t="n">
-        <v>46256</v>
-      </c>
-      <c r="H11" s="35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I11" s="37" t="n">
-        <v>46256</v>
-      </c>
-      <c r="J11" s="36" t="inlineStr">
-        <is>
-          <t>Accountant background; strong financial planning interest</t>
-        </is>
-      </c>
-      <c r="K11" s="37" t="n">
-        <v>46258</v>
-      </c>
-      <c r="L11" s="35" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+      <c r="A11" s="35">
+        <f>IF(B11="","","REC-"&amp;TEXT(11-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B11" s="36" t="inlineStr"/>
+      <c r="C11" s="35" t="inlineStr"/>
+      <c r="D11" s="36" t="inlineStr"/>
+      <c r="E11" s="36" t="inlineStr"/>
+      <c r="F11" s="37" t="n"/>
+      <c r="G11" s="37" t="n"/>
+      <c r="H11" s="35" t="inlineStr"/>
+      <c r="I11" s="37" t="n"/>
+      <c r="J11" s="36" t="inlineStr"/>
+      <c r="K11" s="37" t="n"/>
+      <c r="L11" s="35" t="inlineStr"/>
       <c r="M11" s="37" t="n"/>
-      <c r="N11" s="38" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="O11" s="36" t="inlineStr">
-        <is>
-          <t>Completed 4 of 6 modules</t>
-        </is>
-      </c>
+      <c r="N11" s="38" t="n"/>
+      <c r="O11" s="36" t="inlineStr"/>
       <c r="P11" s="35">
         <f>IF(B11="","",IF(L11="Yes","LMS Completed (Ready for Exam)",IF(L11="In Progress","LMS In Progress",IF(H11="Yes","ADD Attended - Awaiting LMS",IF(H11="Rescheduled","ADD Rescheduled",IF(H11="Pending","ADD Scheduled",IF(H11="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q11" s="36" t="inlineStr">
-        <is>
-          <t>Remind recruit to complete final 2 LMS modules</t>
-        </is>
-      </c>
-      <c r="R11" s="37" t="n">
-        <v>46281</v>
-      </c>
-      <c r="S11" s="36" t="inlineStr">
-        <is>
-          <t>Followed up via WhatsApp; targeting completion this week</t>
-        </is>
-      </c>
+      <c r="Q11" s="36" t="inlineStr"/>
+      <c r="R11" s="37" t="n"/>
+      <c r="S11" s="36" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="39" t="inlineStr">
-        <is>
-          <t>REC-004</t>
-        </is>
-      </c>
-      <c r="B12" s="40" t="inlineStr">
-        <is>
-          <t>Garcia, Patricia Mae</t>
-        </is>
-      </c>
-      <c r="C12" s="39" t="inlineStr">
-        <is>
-          <t>+63 920 456 7890</t>
-        </is>
-      </c>
-      <c r="D12" s="40" t="inlineStr">
-        <is>
-          <t>patricia.garcia@gmail.com</t>
-        </is>
-      </c>
-      <c r="E12" s="40" t="inlineStr">
-        <is>
-          <t>Elena Gomez</t>
-        </is>
-      </c>
-      <c r="F12" s="41" t="n">
-        <v>46254</v>
-      </c>
-      <c r="G12" s="41" t="n">
-        <v>46256</v>
-      </c>
-      <c r="H12" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I12" s="41" t="n">
-        <v>46256</v>
-      </c>
-      <c r="J12" s="40" t="inlineStr">
-        <is>
-          <t>Corporate sales experience; enthusiastic candidate</t>
-        </is>
-      </c>
-      <c r="K12" s="41" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L12" s="39" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+      <c r="A12" s="39">
+        <f>IF(B12="","","REC-"&amp;TEXT(12-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B12" s="40" t="inlineStr"/>
+      <c r="C12" s="39" t="inlineStr"/>
+      <c r="D12" s="40" t="inlineStr"/>
+      <c r="E12" s="40" t="inlineStr"/>
+      <c r="F12" s="41" t="n"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="39" t="inlineStr"/>
+      <c r="I12" s="41" t="n"/>
+      <c r="J12" s="40" t="inlineStr"/>
+      <c r="K12" s="41" t="n"/>
+      <c r="L12" s="39" t="inlineStr"/>
       <c r="M12" s="41" t="n"/>
-      <c r="N12" s="42" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O12" s="40" t="inlineStr">
-        <is>
-          <t>Completed 3 of 6 modules</t>
-        </is>
-      </c>
+      <c r="N12" s="42" t="n"/>
+      <c r="O12" s="40" t="inlineStr"/>
       <c r="P12" s="39">
         <f>IF(B12="","",IF(L12="Yes","LMS Completed (Ready for Exam)",IF(L12="In Progress","LMS In Progress",IF(H12="Yes","ADD Attended - Awaiting LMS",IF(H12="Rescheduled","ADD Rescheduled",IF(H12="Pending","ADD Scheduled",IF(H12="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q12" s="40" t="inlineStr">
-        <is>
-          <t>Follow up on Module 4 (Variable Unit-Linked)</t>
-        </is>
-      </c>
-      <c r="R12" s="41" t="n">
-        <v>46282</v>
-      </c>
-      <c r="S12" s="40" t="inlineStr">
-        <is>
-          <t>Asked clarification about investment funds</t>
-        </is>
-      </c>
+      <c r="Q12" s="40" t="inlineStr"/>
+      <c r="R12" s="41" t="n"/>
+      <c r="S12" s="40" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>REC-005</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="inlineStr">
-        <is>
-          <t>Aquino, Roberto Carlos</t>
-        </is>
-      </c>
-      <c r="C13" s="35" t="inlineStr">
-        <is>
-          <t>+63 921 567 8901</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>roberto.aquino@gmail.com</t>
-        </is>
-      </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>David Tan</t>
-        </is>
-      </c>
-      <c r="F13" s="37" t="n">
-        <v>46259</v>
-      </c>
-      <c r="G13" s="37" t="n">
-        <v>46263</v>
-      </c>
-      <c r="H13" s="35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I13" s="37" t="n">
-        <v>46263</v>
-      </c>
-      <c r="J13" s="36" t="inlineStr">
-        <is>
-          <t>Attended full ADD orientation; signed intention form</t>
-        </is>
-      </c>
-      <c r="K13" s="37" t="n">
-        <v>46266</v>
-      </c>
-      <c r="L13" s="35" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="A13" s="35">
+        <f>IF(B13="","","REC-"&amp;TEXT(13-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B13" s="36" t="inlineStr"/>
+      <c r="C13" s="35" t="inlineStr"/>
+      <c r="D13" s="36" t="inlineStr"/>
+      <c r="E13" s="36" t="inlineStr"/>
+      <c r="F13" s="37" t="n"/>
+      <c r="G13" s="37" t="n"/>
+      <c r="H13" s="35" t="inlineStr"/>
+      <c r="I13" s="37" t="n"/>
+      <c r="J13" s="36" t="inlineStr"/>
+      <c r="K13" s="37" t="n"/>
+      <c r="L13" s="35" t="inlineStr"/>
       <c r="M13" s="37" t="n"/>
-      <c r="N13" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="36" t="inlineStr">
-        <is>
-          <t>Account created, awaiting first login</t>
-        </is>
-      </c>
+      <c r="N13" s="38" t="n"/>
+      <c r="O13" s="36" t="inlineStr"/>
       <c r="P13" s="35">
         <f>IF(B13="","",IF(L13="Yes","LMS Completed (Ready for Exam)",IF(L13="In Progress","LMS In Progress",IF(H13="Yes","ADD Attended - Awaiting LMS",IF(H13="Rescheduled","ADD Rescheduled",IF(H13="Pending","ADD Scheduled",IF(H13="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q13" s="36" t="inlineStr">
-        <is>
-          <t>Send LMS login credentials &amp; quick-start guide</t>
-        </is>
-      </c>
-      <c r="R13" s="37" t="n">
-        <v>46281</v>
-      </c>
-      <c r="S13" s="36" t="inlineStr">
-        <is>
-          <t>Resent activation link to recruit email</t>
-        </is>
-      </c>
+      <c r="Q13" s="36" t="inlineStr"/>
+      <c r="R13" s="37" t="n"/>
+      <c r="S13" s="36" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="39" t="inlineStr">
-        <is>
-          <t>REC-006</t>
-        </is>
-      </c>
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t>Bautista, Sarah Jane</t>
-        </is>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
-        <is>
-          <t>+63 922 678 9012</t>
-        </is>
-      </c>
-      <c r="D14" s="40" t="inlineStr">
-        <is>
-          <t>sarah.bautista@gmail.com</t>
-        </is>
-      </c>
-      <c r="E14" s="40" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins (UM)</t>
-        </is>
-      </c>
-      <c r="F14" s="41" t="n">
-        <v>46260</v>
-      </c>
-      <c r="G14" s="41" t="n">
-        <v>46263</v>
-      </c>
-      <c r="H14" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I14" s="41" t="n">
-        <v>46263</v>
-      </c>
-      <c r="J14" s="40" t="inlineStr">
-        <is>
-          <t>Former bank officer; high potential for rapid onboarding</t>
-        </is>
-      </c>
-      <c r="K14" s="41" t="n">
-        <v>46264</v>
-      </c>
-      <c r="L14" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M14" s="41" t="n">
-        <v>46273</v>
-      </c>
-      <c r="N14" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" s="40" t="inlineStr">
-        <is>
-          <t>Cert #LMS-2026-912 (Passed 96%)</t>
-        </is>
-      </c>
+      <c r="A14" s="39">
+        <f>IF(B14="","","REC-"&amp;TEXT(14-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B14" s="40" t="inlineStr"/>
+      <c r="C14" s="39" t="inlineStr"/>
+      <c r="D14" s="40" t="inlineStr"/>
+      <c r="E14" s="40" t="inlineStr"/>
+      <c r="F14" s="41" t="n"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="39" t="inlineStr"/>
+      <c r="I14" s="41" t="n"/>
+      <c r="J14" s="40" t="inlineStr"/>
+      <c r="K14" s="41" t="n"/>
+      <c r="L14" s="39" t="inlineStr"/>
+      <c r="M14" s="41" t="n"/>
+      <c r="N14" s="42" t="n"/>
+      <c r="O14" s="40" t="inlineStr"/>
       <c r="P14" s="39">
         <f>IF(B14="","",IF(L14="Yes","LMS Completed (Ready for Exam)",IF(L14="In Progress","LMS In Progress",IF(H14="Yes","ADD Attended - Awaiting LMS",IF(H14="Rescheduled","ADD Rescheduled",IF(H14="Pending","ADD Scheduled",IF(H14="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q14" s="40" t="inlineStr">
-        <is>
-          <t>Submit licensing application to agency coordinator</t>
-        </is>
-      </c>
-      <c r="R14" s="41" t="n">
-        <v>46283</v>
-      </c>
-      <c r="S14" s="40" t="inlineStr">
-        <is>
-          <t>Top scorer in batch; ready for branch endorsement</t>
-        </is>
-      </c>
+      <c r="Q14" s="40" t="inlineStr"/>
+      <c r="R14" s="41" t="n"/>
+      <c r="S14" s="40" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>REC-007</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>Mendoza, Christian Paul</t>
-        </is>
-      </c>
-      <c r="C15" s="35" t="inlineStr">
-        <is>
-          <t>+63 923 789 0123</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr">
-        <is>
-          <t>cp.mendoza@gmail.com</t>
-        </is>
-      </c>
-      <c r="E15" s="36" t="inlineStr">
-        <is>
-          <t>Michael Chang</t>
-        </is>
-      </c>
-      <c r="F15" s="37" t="n">
-        <v>46267</v>
-      </c>
-      <c r="G15" s="37" t="n">
-        <v>46284</v>
-      </c>
-      <c r="H15" s="35" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="A15" s="35">
+        <f>IF(B15="","","REC-"&amp;TEXT(15-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B15" s="36" t="inlineStr"/>
+      <c r="C15" s="35" t="inlineStr"/>
+      <c r="D15" s="36" t="inlineStr"/>
+      <c r="E15" s="36" t="inlineStr"/>
+      <c r="F15" s="37" t="n"/>
+      <c r="G15" s="37" t="n"/>
+      <c r="H15" s="35" t="inlineStr"/>
       <c r="I15" s="37" t="n"/>
-      <c r="J15" s="36" t="inlineStr">
-        <is>
-          <t>Confirmed invitation receipt; interested in career preview</t>
-        </is>
-      </c>
+      <c r="J15" s="36" t="inlineStr"/>
       <c r="K15" s="37" t="n"/>
-      <c r="L15" s="35" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="L15" s="35" t="inlineStr"/>
       <c r="M15" s="37" t="n"/>
-      <c r="N15" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="36" t="inlineStr">
-        <is>
-          <t>Pending ADD completion</t>
-        </is>
-      </c>
+      <c r="N15" s="38" t="n"/>
+      <c r="O15" s="36" t="inlineStr"/>
       <c r="P15" s="35">
         <f>IF(B15="","",IF(L15="Yes","LMS Completed (Ready for Exam)",IF(L15="In Progress","LMS In Progress",IF(H15="Yes","ADD Attended - Awaiting LMS",IF(H15="Rescheduled","ADD Rescheduled",IF(H15="Pending","ADD Scheduled",IF(H15="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q15" s="36" t="inlineStr">
-        <is>
-          <t>Send ADD webinar link &amp; preparation checklist</t>
-        </is>
-      </c>
-      <c r="R15" s="37" t="n">
-        <v>46283</v>
-      </c>
-      <c r="S15" s="36" t="inlineStr">
-        <is>
-          <t>Referred by Juan Dela Cruz; high enthusiasm</t>
-        </is>
-      </c>
+      <c r="Q15" s="36" t="inlineStr"/>
+      <c r="R15" s="37" t="n"/>
+      <c r="S15" s="36" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="39" t="inlineStr">
-        <is>
-          <t>REC-008</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>Villanueva, Kristine Joy</t>
-        </is>
-      </c>
-      <c r="C16" s="39" t="inlineStr">
-        <is>
-          <t>+63 924 890 1234</t>
-        </is>
-      </c>
-      <c r="D16" s="40" t="inlineStr">
-        <is>
-          <t>kristine.v@yahoo.com</t>
-        </is>
-      </c>
-      <c r="E16" s="40" t="inlineStr">
-        <is>
-          <t>Elena Gomez</t>
-        </is>
-      </c>
-      <c r="F16" s="41" t="n">
-        <v>46266</v>
-      </c>
-      <c r="G16" s="41" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H16" s="39" t="inlineStr">
-        <is>
-          <t>Rescheduled</t>
-        </is>
-      </c>
+      <c r="A16" s="39">
+        <f>IF(B16="","","REC-"&amp;TEXT(16-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B16" s="40" t="inlineStr"/>
+      <c r="C16" s="39" t="inlineStr"/>
+      <c r="D16" s="40" t="inlineStr"/>
+      <c r="E16" s="40" t="inlineStr"/>
+      <c r="F16" s="41" t="n"/>
+      <c r="G16" s="41" t="n"/>
+      <c r="H16" s="39" t="inlineStr"/>
       <c r="I16" s="41" t="n"/>
-      <c r="J16" s="40" t="inlineStr">
-        <is>
-          <t>Family matter on Sept 5; requested transfer to Sept 19</t>
-        </is>
-      </c>
+      <c r="J16" s="40" t="inlineStr"/>
       <c r="K16" s="41" t="n"/>
-      <c r="L16" s="39" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="L16" s="39" t="inlineStr"/>
       <c r="M16" s="41" t="n"/>
-      <c r="N16" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="40" t="inlineStr">
-        <is>
-          <t>Pending ADD completion</t>
-        </is>
-      </c>
+      <c r="N16" s="42" t="n"/>
+      <c r="O16" s="40" t="inlineStr"/>
       <c r="P16" s="39">
         <f>IF(B16="","",IF(L16="Yes","LMS Completed (Ready for Exam)",IF(L16="In Progress","LMS In Progress",IF(H16="Yes","ADD Attended - Awaiting LMS",IF(H16="Rescheduled","ADD Rescheduled",IF(H16="Pending","ADD Scheduled",IF(H16="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q16" s="40" t="inlineStr">
-        <is>
-          <t>Confirm attendance for Sept 19 ADD session</t>
-        </is>
-      </c>
-      <c r="R16" s="41" t="n">
-        <v>46282</v>
-      </c>
-      <c r="S16" s="40" t="inlineStr">
-        <is>
-          <t>Sent updated calendar invite</t>
-        </is>
-      </c>
+      <c r="Q16" s="40" t="inlineStr"/>
+      <c r="R16" s="41" t="n"/>
+      <c r="S16" s="40" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="35" t="inlineStr">
-        <is>
-          <t>REC-009</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="inlineStr">
-        <is>
-          <t>Tan, Michael Angelo</t>
-        </is>
-      </c>
-      <c r="C17" s="35" t="inlineStr">
-        <is>
-          <t>+63 925 901 2345</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr">
-        <is>
-          <t>mike.tan@hotmail.com</t>
-        </is>
-      </c>
-      <c r="E17" s="36" t="inlineStr">
-        <is>
-          <t>Michael Chang</t>
-        </is>
-      </c>
-      <c r="F17" s="37" t="n">
-        <v>46268</v>
-      </c>
-      <c r="G17" s="37" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H17" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A17" s="35">
+        <f>IF(B17="","","REC-"&amp;TEXT(17-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B17" s="36" t="inlineStr"/>
+      <c r="C17" s="35" t="inlineStr"/>
+      <c r="D17" s="36" t="inlineStr"/>
+      <c r="E17" s="36" t="inlineStr"/>
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="37" t="n"/>
+      <c r="H17" s="35" t="inlineStr"/>
       <c r="I17" s="37" t="n"/>
-      <c r="J17" s="36" t="inlineStr">
-        <is>
-          <t>No-show; phone was unattended during call time</t>
-        </is>
-      </c>
+      <c r="J17" s="36" t="inlineStr"/>
       <c r="K17" s="37" t="n"/>
-      <c r="L17" s="35" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="L17" s="35" t="inlineStr"/>
       <c r="M17" s="37" t="n"/>
-      <c r="N17" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="36" t="inlineStr">
-        <is>
-          <t>Pending ADD re-engagement</t>
-        </is>
-      </c>
+      <c r="N17" s="38" t="n"/>
+      <c r="O17" s="36" t="inlineStr"/>
       <c r="P17" s="35">
         <f>IF(B17="","",IF(L17="Yes","LMS Completed (Ready for Exam)",IF(L17="In Progress","LMS In Progress",IF(H17="Yes","ADD Attended - Awaiting LMS",IF(H17="Rescheduled","ADD Rescheduled",IF(H17="Pending","ADD Scheduled",IF(H17="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q17" s="36" t="inlineStr">
-        <is>
-          <t>Call back and re-invite to next ADD session</t>
-        </is>
-      </c>
-      <c r="R17" s="37" t="n">
-        <v>46281</v>
-      </c>
-      <c r="S17" s="36" t="inlineStr">
-        <is>
-          <t>Sent follow-up email with recording preview</t>
-        </is>
-      </c>
+      <c r="Q17" s="36" t="inlineStr"/>
+      <c r="R17" s="37" t="n"/>
+      <c r="S17" s="36" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="39" t="inlineStr">
-        <is>
-          <t>REC-010</t>
-        </is>
-      </c>
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>Ramos, Beatrice Nicole</t>
-        </is>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>+63 926 012 3456</t>
-        </is>
-      </c>
-      <c r="D18" s="40" t="inlineStr">
-        <is>
-          <t>beatrice.ramos@gmail.com</t>
-        </is>
-      </c>
-      <c r="E18" s="40" t="inlineStr">
-        <is>
-          <t>David Tan</t>
-        </is>
-      </c>
-      <c r="F18" s="41" t="n">
-        <v>46262</v>
-      </c>
-      <c r="G18" s="41" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H18" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I18" s="41" t="n">
-        <v>46270</v>
-      </c>
-      <c r="J18" s="40" t="inlineStr">
-        <is>
-          <t>Very interactive; asked about commission &amp; team structure</t>
-        </is>
-      </c>
-      <c r="K18" s="41" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L18" s="39" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+      <c r="A18" s="39">
+        <f>IF(B18="","","REC-"&amp;TEXT(18-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B18" s="40" t="inlineStr"/>
+      <c r="C18" s="39" t="inlineStr"/>
+      <c r="D18" s="40" t="inlineStr"/>
+      <c r="E18" s="40" t="inlineStr"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="39" t="inlineStr"/>
+      <c r="I18" s="41" t="n"/>
+      <c r="J18" s="40" t="inlineStr"/>
+      <c r="K18" s="41" t="n"/>
+      <c r="L18" s="39" t="inlineStr"/>
       <c r="M18" s="41" t="n"/>
-      <c r="N18" s="42" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="O18" s="40" t="inlineStr">
-        <is>
-          <t>Completed 2 of 6 modules</t>
-        </is>
-      </c>
+      <c r="N18" s="42" t="n"/>
+      <c r="O18" s="40" t="inlineStr"/>
       <c r="P18" s="39">
         <f>IF(B18="","",IF(L18="Yes","LMS Completed (Ready for Exam)",IF(L18="In Progress","LMS In Progress",IF(H18="Yes","ADD Attended - Awaiting LMS",IF(H18="Rescheduled","ADD Rescheduled",IF(H18="Pending","ADD Scheduled",IF(H18="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q18" s="40" t="inlineStr">
-        <is>
-          <t>Check if needing technical assistance on portal</t>
-        </is>
-      </c>
-      <c r="R18" s="41" t="n">
-        <v>46282</v>
-      </c>
-      <c r="S18" s="40" t="inlineStr">
-        <is>
-          <t>Reported video playback lag; advised to use Chrome</t>
-        </is>
-      </c>
+      <c r="Q18" s="40" t="inlineStr"/>
+      <c r="R18" s="41" t="n"/>
+      <c r="S18" s="40" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="35" t="inlineStr">
-        <is>
-          <t>REC-011</t>
-        </is>
-      </c>
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>Castro, Jonathan David</t>
-        </is>
-      </c>
-      <c r="C19" s="35" t="inlineStr">
-        <is>
-          <t>+63 927 123 4568</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
-        <is>
-          <t>jdcastro@gmail.com</t>
-        </is>
-      </c>
-      <c r="E19" s="36" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins (UM)</t>
-        </is>
-      </c>
-      <c r="F19" s="37" t="n">
-        <v>46256</v>
-      </c>
-      <c r="G19" s="37" t="n">
-        <v>46263</v>
-      </c>
-      <c r="H19" s="35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I19" s="37" t="n">
-        <v>46263</v>
-      </c>
-      <c r="J19" s="36" t="inlineStr">
-        <is>
-          <t>Strong communication skills; completed onboarding docs</t>
-        </is>
-      </c>
-      <c r="K19" s="37" t="n">
-        <v>46265</v>
-      </c>
-      <c r="L19" s="35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M19" s="37" t="n">
-        <v>46274</v>
-      </c>
-      <c r="N19" s="38" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="36" t="inlineStr">
-        <is>
-          <t>Cert #LMS-2026-928 (Passed 91%)</t>
-        </is>
-      </c>
+      <c r="A19" s="35">
+        <f>IF(B19="","","REC-"&amp;TEXT(19-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B19" s="36" t="inlineStr"/>
+      <c r="C19" s="35" t="inlineStr"/>
+      <c r="D19" s="36" t="inlineStr"/>
+      <c r="E19" s="36" t="inlineStr"/>
+      <c r="F19" s="37" t="n"/>
+      <c r="G19" s="37" t="n"/>
+      <c r="H19" s="35" t="inlineStr"/>
+      <c r="I19" s="37" t="n"/>
+      <c r="J19" s="36" t="inlineStr"/>
+      <c r="K19" s="37" t="n"/>
+      <c r="L19" s="35" t="inlineStr"/>
+      <c r="M19" s="37" t="n"/>
+      <c r="N19" s="38" t="n"/>
+      <c r="O19" s="36" t="inlineStr"/>
       <c r="P19" s="35">
         <f>IF(B19="","",IF(L19="Yes","LMS Completed (Ready for Exam)",IF(L19="In Progress","LMS In Progress",IF(H19="Yes","ADD Attended - Awaiting LMS",IF(H19="Rescheduled","ADD Rescheduled",IF(H19="Pending","ADD Scheduled",IF(H19="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q19" s="36" t="inlineStr">
-        <is>
-          <t>Endorse for IC Exam and schedule branch orientation</t>
-        </is>
-      </c>
-      <c r="R19" s="37" t="n">
-        <v>46284</v>
-      </c>
-      <c r="S19" s="36" t="inlineStr">
-        <is>
-          <t>Exam fee receipt confirmed</t>
-        </is>
-      </c>
+      <c r="Q19" s="36" t="inlineStr"/>
+      <c r="R19" s="37" t="n"/>
+      <c r="S19" s="36" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="39" t="inlineStr">
-        <is>
-          <t>REC-012</t>
-        </is>
-      </c>
-      <c r="B20" s="40" t="inlineStr">
-        <is>
-          <t>Navarro, Angela Marie</t>
-        </is>
-      </c>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>+63 928 234 5679</t>
-        </is>
-      </c>
-      <c r="D20" s="40" t="inlineStr">
-        <is>
-          <t>angela.navarro@gmail.com</t>
-        </is>
-      </c>
-      <c r="E20" s="40" t="inlineStr">
-        <is>
-          <t>Elena Gomez</t>
-        </is>
-      </c>
-      <c r="F20" s="41" t="n">
-        <v>46273</v>
-      </c>
-      <c r="G20" s="41" t="n">
-        <v>46284</v>
-      </c>
-      <c r="H20" s="39" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="A20" s="39">
+        <f>IF(B20="","","REC-"&amp;TEXT(20-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B20" s="40" t="inlineStr"/>
+      <c r="C20" s="39" t="inlineStr"/>
+      <c r="D20" s="40" t="inlineStr"/>
+      <c r="E20" s="40" t="inlineStr"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="39" t="inlineStr"/>
       <c r="I20" s="41" t="n"/>
-      <c r="J20" s="40" t="inlineStr">
-        <is>
-          <t>Expressed interest in flexible part-time income</t>
-        </is>
-      </c>
+      <c r="J20" s="40" t="inlineStr"/>
       <c r="K20" s="41" t="n"/>
-      <c r="L20" s="39" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="L20" s="39" t="inlineStr"/>
       <c r="M20" s="41" t="n"/>
-      <c r="N20" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="40" t="inlineStr">
-        <is>
-          <t>Pending ADD completion</t>
-        </is>
-      </c>
+      <c r="N20" s="42" t="n"/>
+      <c r="O20" s="40" t="inlineStr"/>
       <c r="P20" s="39">
         <f>IF(B20="","",IF(L20="Yes","LMS Completed (Ready for Exam)",IF(L20="In Progress","LMS In Progress",IF(H20="Yes","ADD Attended - Awaiting LMS",IF(H20="Rescheduled","ADD Rescheduled",IF(H20="Pending","ADD Scheduled",IF(H20="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q20" s="40" t="inlineStr">
-        <is>
-          <t>Follow up RSVP for upcoming ADD orientation</t>
-        </is>
-      </c>
-      <c r="R20" s="41" t="n">
-        <v>46283</v>
-      </c>
-      <c r="S20" s="40" t="inlineStr">
-        <is>
-          <t>Messaged on LinkedIn; follow up tomorrow</t>
-        </is>
-      </c>
+      <c r="Q20" s="40" t="inlineStr"/>
+      <c r="R20" s="41" t="n"/>
+      <c r="S20" s="40" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="35" t="inlineStr">
-        <is>
-          <t>REC-013</t>
-        </is>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>Lim, Gabriel Francis</t>
-        </is>
-      </c>
-      <c r="C21" s="35" t="inlineStr">
-        <is>
-          <t>+63 929 345 6780</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="inlineStr">
-        <is>
-          <t>gabriel.lim@gmail.com</t>
-        </is>
-      </c>
-      <c r="E21" s="36" t="inlineStr">
-        <is>
-          <t>Michael Chang</t>
-        </is>
-      </c>
-      <c r="F21" s="37" t="n">
-        <v>46264</v>
-      </c>
-      <c r="G21" s="37" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H21" s="35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I21" s="37" t="n">
-        <v>46270</v>
-      </c>
-      <c r="J21" s="36" t="inlineStr">
-        <is>
-          <t>Attended ADD; completed career interest profiling</t>
-        </is>
-      </c>
-      <c r="K21" s="37" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L21" s="35" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="A21" s="35">
+        <f>IF(B21="","","REC-"&amp;TEXT(21-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B21" s="36" t="inlineStr"/>
+      <c r="C21" s="35" t="inlineStr"/>
+      <c r="D21" s="36" t="inlineStr"/>
+      <c r="E21" s="36" t="inlineStr"/>
+      <c r="F21" s="37" t="n"/>
+      <c r="G21" s="37" t="n"/>
+      <c r="H21" s="35" t="inlineStr"/>
+      <c r="I21" s="37" t="n"/>
+      <c r="J21" s="36" t="inlineStr"/>
+      <c r="K21" s="37" t="n"/>
+      <c r="L21" s="35" t="inlineStr"/>
       <c r="M21" s="37" t="n"/>
-      <c r="N21" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="36" t="inlineStr">
-        <is>
-          <t>Credentials issued 09/08</t>
-        </is>
-      </c>
+      <c r="N21" s="38" t="n"/>
+      <c r="O21" s="36" t="inlineStr"/>
       <c r="P21" s="35">
         <f>IF(B21="","",IF(L21="Yes","LMS Completed (Ready for Exam)",IF(L21="In Progress","LMS In Progress",IF(H21="Yes","ADD Attended - Awaiting LMS",IF(H21="Rescheduled","ADD Rescheduled",IF(H21="Pending","ADD Scheduled",IF(H21="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q21" s="36" t="inlineStr">
-        <is>
-          <t>Check why LMS has not been started after 1 week</t>
-        </is>
-      </c>
-      <c r="R21" s="37" t="n">
-        <v>46281</v>
-      </c>
-      <c r="S21" s="36" t="inlineStr">
-        <is>
-          <t>Candidate busy with work deadline; starts Saturday</t>
-        </is>
-      </c>
+      <c r="Q21" s="36" t="inlineStr"/>
+      <c r="R21" s="37" t="n"/>
+      <c r="S21" s="36" t="inlineStr"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="39" t="inlineStr">
-        <is>
-          <t>REC-014</t>
-        </is>
-      </c>
-      <c r="B22" s="40" t="inlineStr">
-        <is>
-          <t>Flores, Camille Sophia</t>
-        </is>
-      </c>
-      <c r="C22" s="39" t="inlineStr">
-        <is>
-          <t>+63 930 456 7891</t>
-        </is>
-      </c>
-      <c r="D22" s="40" t="inlineStr">
-        <is>
-          <t>camille.flores@gmail.com</t>
-        </is>
-      </c>
-      <c r="E22" s="40" t="inlineStr">
-        <is>
-          <t>David Tan</t>
-        </is>
-      </c>
-      <c r="F22" s="41" t="n">
-        <v>46263</v>
-      </c>
-      <c r="G22" s="41" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H22" s="39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I22" s="41" t="n">
-        <v>46270</v>
-      </c>
-      <c r="J22" s="40" t="inlineStr">
-        <is>
-          <t>Educator transitioning to financial services industry</t>
-        </is>
-      </c>
-      <c r="K22" s="41" t="n">
-        <v>46271</v>
-      </c>
-      <c r="L22" s="39" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
+      <c r="A22" s="39">
+        <f>IF(B22="","","REC-"&amp;TEXT(22-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B22" s="40" t="inlineStr"/>
+      <c r="C22" s="39" t="inlineStr"/>
+      <c r="D22" s="40" t="inlineStr"/>
+      <c r="E22" s="40" t="inlineStr"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="39" t="inlineStr"/>
+      <c r="I22" s="41" t="n"/>
+      <c r="J22" s="40" t="inlineStr"/>
+      <c r="K22" s="41" t="n"/>
+      <c r="L22" s="39" t="inlineStr"/>
       <c r="M22" s="41" t="n"/>
-      <c r="N22" s="42" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="O22" s="40" t="inlineStr">
-        <is>
-          <t>Completed 5 of 6 modules</t>
-        </is>
-      </c>
+      <c r="N22" s="42" t="n"/>
+      <c r="O22" s="40" t="inlineStr"/>
       <c r="P22" s="39">
         <f>IF(B22="","",IF(L22="Yes","LMS Completed (Ready for Exam)",IF(L22="In Progress","LMS In Progress",IF(H22="Yes","ADD Attended - Awaiting LMS",IF(H22="Rescheduled","ADD Rescheduled",IF(H22="Pending","ADD Scheduled",IF(H22="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q22" s="40" t="inlineStr">
-        <is>
-          <t>Remind recruit to submit practice mock exam</t>
-        </is>
-      </c>
-      <c r="R22" s="41" t="n">
-        <v>46281</v>
-      </c>
-      <c r="S22" s="40" t="inlineStr">
-        <is>
-          <t>Targeting final module completion tonight</t>
-        </is>
-      </c>
+      <c r="Q22" s="40" t="inlineStr"/>
+      <c r="R22" s="41" t="n"/>
+      <c r="S22" s="40" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="35" t="inlineStr">
-        <is>
-          <t>REC-015</t>
-        </is>
-      </c>
-      <c r="B23" s="36" t="inlineStr">
-        <is>
-          <t>Diaz, Vincent Edward</t>
-        </is>
-      </c>
-      <c r="C23" s="35" t="inlineStr">
-        <is>
-          <t>+63 931 567 8902</t>
-        </is>
-      </c>
-      <c r="D23" s="36" t="inlineStr">
-        <is>
-          <t>vincent.diaz@gmail.com</t>
-        </is>
-      </c>
-      <c r="E23" s="36" t="inlineStr">
-        <is>
-          <t>Elena Gomez</t>
-        </is>
-      </c>
-      <c r="F23" s="37" t="n">
-        <v>46269</v>
-      </c>
-      <c r="G23" s="37" t="n">
-        <v>46277</v>
-      </c>
-      <c r="H23" s="35" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A23" s="35">
+        <f>IF(B23="","","REC-"&amp;TEXT(23-8,"000"))</f>
+        <v/>
+      </c>
+      <c r="B23" s="36" t="inlineStr"/>
+      <c r="C23" s="35" t="inlineStr"/>
+      <c r="D23" s="36" t="inlineStr"/>
+      <c r="E23" s="36" t="inlineStr"/>
+      <c r="F23" s="37" t="n"/>
+      <c r="G23" s="37" t="n"/>
+      <c r="H23" s="35" t="inlineStr"/>
       <c r="I23" s="37" t="n"/>
-      <c r="J23" s="36" t="inlineStr">
-        <is>
-          <t>Unforeseen overtime work; could not attend ADD</t>
-        </is>
-      </c>
+      <c r="J23" s="36" t="inlineStr"/>
       <c r="K23" s="37" t="n"/>
-      <c r="L23" s="35" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+      <c r="L23" s="35" t="inlineStr"/>
       <c r="M23" s="37" t="n"/>
-      <c r="N23" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="36" t="inlineStr">
-        <is>
-          <t>Pending ADD re-engagement</t>
-        </is>
-      </c>
+      <c r="N23" s="38" t="n"/>
+      <c r="O23" s="36" t="inlineStr"/>
       <c r="P23" s="35">
         <f>IF(B23="","",IF(L23="Yes","LMS Completed (Ready for Exam)",IF(L23="In Progress","LMS In Progress",IF(H23="Yes","ADD Attended - Awaiting LMS",IF(H23="Rescheduled","ADD Rescheduled",IF(H23="Pending","ADD Scheduled",IF(H23="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q23" s="36" t="inlineStr">
-        <is>
-          <t>Offer weekend 1-on-1 career briefing or video</t>
-        </is>
-      </c>
-      <c r="R23" s="37" t="n">
-        <v>46282</v>
-      </c>
-      <c r="S23" s="36" t="inlineStr">
-        <is>
-          <t>Prefers Saturday morning slot</t>
-        </is>
-      </c>
+      <c r="Q23" s="36" t="inlineStr"/>
+      <c r="R23" s="37" t="n"/>
+      <c r="S23" s="36" t="inlineStr"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="39">
         <f>IF(B24="","","REC-"&amp;TEXT(24-8,"000"))</f>
         <v/>
       </c>
-      <c r="B24" s="40" t="n"/>
-      <c r="C24" s="39" t="n"/>
-      <c r="D24" s="40" t="n"/>
-      <c r="E24" s="40" t="n"/>
+      <c r="B24" s="40" t="inlineStr"/>
+      <c r="C24" s="39" t="inlineStr"/>
+      <c r="D24" s="40" t="inlineStr"/>
+      <c r="E24" s="40" t="inlineStr"/>
       <c r="F24" s="41" t="n"/>
       <c r="G24" s="41" t="n"/>
-      <c r="H24" s="39" t="n"/>
+      <c r="H24" s="39" t="inlineStr"/>
       <c r="I24" s="41" t="n"/>
-      <c r="J24" s="40" t="n"/>
+      <c r="J24" s="40" t="inlineStr"/>
       <c r="K24" s="41" t="n"/>
-      <c r="L24" s="39" t="n"/>
+      <c r="L24" s="39" t="inlineStr"/>
       <c r="M24" s="41" t="n"/>
       <c r="N24" s="42" t="n"/>
-      <c r="O24" s="40" t="n"/>
+      <c r="O24" s="40" t="inlineStr"/>
       <c r="P24" s="39">
         <f>IF(B24="","",IF(L24="Yes","LMS Completed (Ready for Exam)",IF(L24="In Progress","LMS In Progress",IF(H24="Yes","ADD Attended - Awaiting LMS",IF(H24="Rescheduled","ADD Rescheduled",IF(H24="Pending","ADD Scheduled",IF(H24="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q24" s="40" t="n"/>
+      <c r="Q24" s="40" t="inlineStr"/>
       <c r="R24" s="41" t="n"/>
-      <c r="S24" s="40" t="n"/>
+      <c r="S24" s="40" t="inlineStr"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="35">
         <f>IF(B25="","","REC-"&amp;TEXT(25-8,"000"))</f>
         <v/>
       </c>
-      <c r="B25" s="36" t="n"/>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
+      <c r="B25" s="36" t="inlineStr"/>
+      <c r="C25" s="35" t="inlineStr"/>
+      <c r="D25" s="36" t="inlineStr"/>
+      <c r="E25" s="36" t="inlineStr"/>
       <c r="F25" s="37" t="n"/>
       <c r="G25" s="37" t="n"/>
-      <c r="H25" s="35" t="n"/>
+      <c r="H25" s="35" t="inlineStr"/>
       <c r="I25" s="37" t="n"/>
-      <c r="J25" s="36" t="n"/>
+      <c r="J25" s="36" t="inlineStr"/>
       <c r="K25" s="37" t="n"/>
-      <c r="L25" s="35" t="n"/>
+      <c r="L25" s="35" t="inlineStr"/>
       <c r="M25" s="37" t="n"/>
       <c r="N25" s="38" t="n"/>
-      <c r="O25" s="36" t="n"/>
+      <c r="O25" s="36" t="inlineStr"/>
       <c r="P25" s="35">
         <f>IF(B25="","",IF(L25="Yes","LMS Completed (Ready for Exam)",IF(L25="In Progress","LMS In Progress",IF(H25="Yes","ADD Attended - Awaiting LMS",IF(H25="Rescheduled","ADD Rescheduled",IF(H25="Pending","ADD Scheduled",IF(H25="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q25" s="36" t="n"/>
+      <c r="Q25" s="36" t="inlineStr"/>
       <c r="R25" s="37" t="n"/>
-      <c r="S25" s="36" t="n"/>
+      <c r="S25" s="36" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="39">
         <f>IF(B26="","","REC-"&amp;TEXT(26-8,"000"))</f>
         <v/>
       </c>
-      <c r="B26" s="40" t="n"/>
-      <c r="C26" s="39" t="n"/>
-      <c r="D26" s="40" t="n"/>
-      <c r="E26" s="40" t="n"/>
+      <c r="B26" s="40" t="inlineStr"/>
+      <c r="C26" s="39" t="inlineStr"/>
+      <c r="D26" s="40" t="inlineStr"/>
+      <c r="E26" s="40" t="inlineStr"/>
       <c r="F26" s="41" t="n"/>
       <c r="G26" s="41" t="n"/>
-      <c r="H26" s="39" t="n"/>
+      <c r="H26" s="39" t="inlineStr"/>
       <c r="I26" s="41" t="n"/>
-      <c r="J26" s="40" t="n"/>
+      <c r="J26" s="40" t="inlineStr"/>
       <c r="K26" s="41" t="n"/>
-      <c r="L26" s="39" t="n"/>
+      <c r="L26" s="39" t="inlineStr"/>
       <c r="M26" s="41" t="n"/>
       <c r="N26" s="42" t="n"/>
-      <c r="O26" s="40" t="n"/>
+      <c r="O26" s="40" t="inlineStr"/>
       <c r="P26" s="39">
         <f>IF(B26="","",IF(L26="Yes","LMS Completed (Ready for Exam)",IF(L26="In Progress","LMS In Progress",IF(H26="Yes","ADD Attended - Awaiting LMS",IF(H26="Rescheduled","ADD Rescheduled",IF(H26="Pending","ADD Scheduled",IF(H26="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q26" s="40" t="n"/>
+      <c r="Q26" s="40" t="inlineStr"/>
       <c r="R26" s="41" t="n"/>
-      <c r="S26" s="40" t="n"/>
+      <c r="S26" s="40" t="inlineStr"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="35">
         <f>IF(B27="","","REC-"&amp;TEXT(27-8,"000"))</f>
         <v/>
       </c>
-      <c r="B27" s="36" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
+      <c r="B27" s="36" t="inlineStr"/>
+      <c r="C27" s="35" t="inlineStr"/>
+      <c r="D27" s="36" t="inlineStr"/>
+      <c r="E27" s="36" t="inlineStr"/>
       <c r="F27" s="37" t="n"/>
       <c r="G27" s="37" t="n"/>
-      <c r="H27" s="35" t="n"/>
+      <c r="H27" s="35" t="inlineStr"/>
       <c r="I27" s="37" t="n"/>
-      <c r="J27" s="36" t="n"/>
+      <c r="J27" s="36" t="inlineStr"/>
       <c r="K27" s="37" t="n"/>
-      <c r="L27" s="35" t="n"/>
+      <c r="L27" s="35" t="inlineStr"/>
       <c r="M27" s="37" t="n"/>
       <c r="N27" s="38" t="n"/>
-      <c r="O27" s="36" t="n"/>
+      <c r="O27" s="36" t="inlineStr"/>
       <c r="P27" s="35">
         <f>IF(B27="","",IF(L27="Yes","LMS Completed (Ready for Exam)",IF(L27="In Progress","LMS In Progress",IF(H27="Yes","ADD Attended - Awaiting LMS",IF(H27="Rescheduled","ADD Rescheduled",IF(H27="Pending","ADD Scheduled",IF(H27="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q27" s="36" t="n"/>
+      <c r="Q27" s="36" t="inlineStr"/>
       <c r="R27" s="37" t="n"/>
-      <c r="S27" s="36" t="n"/>
+      <c r="S27" s="36" t="inlineStr"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="39">
         <f>IF(B28="","","REC-"&amp;TEXT(28-8,"000"))</f>
         <v/>
       </c>
-      <c r="B28" s="40" t="n"/>
-      <c r="C28" s="39" t="n"/>
-      <c r="D28" s="40" t="n"/>
-      <c r="E28" s="40" t="n"/>
+      <c r="B28" s="40" t="inlineStr"/>
+      <c r="C28" s="39" t="inlineStr"/>
+      <c r="D28" s="40" t="inlineStr"/>
+      <c r="E28" s="40" t="inlineStr"/>
       <c r="F28" s="41" t="n"/>
       <c r="G28" s="41" t="n"/>
-      <c r="H28" s="39" t="n"/>
+      <c r="H28" s="39" t="inlineStr"/>
       <c r="I28" s="41" t="n"/>
-      <c r="J28" s="40" t="n"/>
+      <c r="J28" s="40" t="inlineStr"/>
       <c r="K28" s="41" t="n"/>
-      <c r="L28" s="39" t="n"/>
+      <c r="L28" s="39" t="inlineStr"/>
       <c r="M28" s="41" t="n"/>
       <c r="N28" s="42" t="n"/>
-      <c r="O28" s="40" t="n"/>
+      <c r="O28" s="40" t="inlineStr"/>
       <c r="P28" s="39">
         <f>IF(B28="","",IF(L28="Yes","LMS Completed (Ready for Exam)",IF(L28="In Progress","LMS In Progress",IF(H28="Yes","ADD Attended - Awaiting LMS",IF(H28="Rescheduled","ADD Rescheduled",IF(H28="Pending","ADD Scheduled",IF(H28="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q28" s="40" t="n"/>
+      <c r="Q28" s="40" t="inlineStr"/>
       <c r="R28" s="41" t="n"/>
-      <c r="S28" s="40" t="n"/>
+      <c r="S28" s="40" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="35">
         <f>IF(B29="","","REC-"&amp;TEXT(29-8,"000"))</f>
         <v/>
       </c>
-      <c r="B29" s="36" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="36" t="n"/>
+      <c r="B29" s="36" t="inlineStr"/>
+      <c r="C29" s="35" t="inlineStr"/>
+      <c r="D29" s="36" t="inlineStr"/>
+      <c r="E29" s="36" t="inlineStr"/>
       <c r="F29" s="37" t="n"/>
       <c r="G29" s="37" t="n"/>
-      <c r="H29" s="35" t="n"/>
+      <c r="H29" s="35" t="inlineStr"/>
       <c r="I29" s="37" t="n"/>
-      <c r="J29" s="36" t="n"/>
+      <c r="J29" s="36" t="inlineStr"/>
       <c r="K29" s="37" t="n"/>
-      <c r="L29" s="35" t="n"/>
+      <c r="L29" s="35" t="inlineStr"/>
       <c r="M29" s="37" t="n"/>
       <c r="N29" s="38" t="n"/>
-      <c r="O29" s="36" t="n"/>
+      <c r="O29" s="36" t="inlineStr"/>
       <c r="P29" s="35">
         <f>IF(B29="","",IF(L29="Yes","LMS Completed (Ready for Exam)",IF(L29="In Progress","LMS In Progress",IF(H29="Yes","ADD Attended - Awaiting LMS",IF(H29="Rescheduled","ADD Rescheduled",IF(H29="Pending","ADD Scheduled",IF(H29="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q29" s="36" t="n"/>
+      <c r="Q29" s="36" t="inlineStr"/>
       <c r="R29" s="37" t="n"/>
-      <c r="S29" s="36" t="n"/>
+      <c r="S29" s="36" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="39">
         <f>IF(B30="","","REC-"&amp;TEXT(30-8,"000"))</f>
         <v/>
       </c>
-      <c r="B30" s="40" t="n"/>
-      <c r="C30" s="39" t="n"/>
-      <c r="D30" s="40" t="n"/>
-      <c r="E30" s="40" t="n"/>
+      <c r="B30" s="40" t="inlineStr"/>
+      <c r="C30" s="39" t="inlineStr"/>
+      <c r="D30" s="40" t="inlineStr"/>
+      <c r="E30" s="40" t="inlineStr"/>
       <c r="F30" s="41" t="n"/>
       <c r="G30" s="41" t="n"/>
-      <c r="H30" s="39" t="n"/>
+      <c r="H30" s="39" t="inlineStr"/>
       <c r="I30" s="41" t="n"/>
-      <c r="J30" s="40" t="n"/>
+      <c r="J30" s="40" t="inlineStr"/>
       <c r="K30" s="41" t="n"/>
-      <c r="L30" s="39" t="n"/>
+      <c r="L30" s="39" t="inlineStr"/>
       <c r="M30" s="41" t="n"/>
       <c r="N30" s="42" t="n"/>
-      <c r="O30" s="40" t="n"/>
+      <c r="O30" s="40" t="inlineStr"/>
       <c r="P30" s="39">
         <f>IF(B30="","",IF(L30="Yes","LMS Completed (Ready for Exam)",IF(L30="In Progress","LMS In Progress",IF(H30="Yes","ADD Attended - Awaiting LMS",IF(H30="Rescheduled","ADD Rescheduled",IF(H30="Pending","ADD Scheduled",IF(H30="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q30" s="40" t="n"/>
+      <c r="Q30" s="40" t="inlineStr"/>
       <c r="R30" s="41" t="n"/>
-      <c r="S30" s="40" t="n"/>
+      <c r="S30" s="40" t="inlineStr"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="35">
         <f>IF(B31="","","REC-"&amp;TEXT(31-8,"000"))</f>
         <v/>
       </c>
-      <c r="B31" s="36" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
+      <c r="B31" s="36" t="inlineStr"/>
+      <c r="C31" s="35" t="inlineStr"/>
+      <c r="D31" s="36" t="inlineStr"/>
+      <c r="E31" s="36" t="inlineStr"/>
       <c r="F31" s="37" t="n"/>
       <c r="G31" s="37" t="n"/>
-      <c r="H31" s="35" t="n"/>
+      <c r="H31" s="35" t="inlineStr"/>
       <c r="I31" s="37" t="n"/>
-      <c r="J31" s="36" t="n"/>
+      <c r="J31" s="36" t="inlineStr"/>
       <c r="K31" s="37" t="n"/>
-      <c r="L31" s="35" t="n"/>
+      <c r="L31" s="35" t="inlineStr"/>
       <c r="M31" s="37" t="n"/>
       <c r="N31" s="38" t="n"/>
-      <c r="O31" s="36" t="n"/>
+      <c r="O31" s="36" t="inlineStr"/>
       <c r="P31" s="35">
         <f>IF(B31="","",IF(L31="Yes","LMS Completed (Ready for Exam)",IF(L31="In Progress","LMS In Progress",IF(H31="Yes","ADD Attended - Awaiting LMS",IF(H31="Rescheduled","ADD Rescheduled",IF(H31="Pending","ADD Scheduled",IF(H31="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q31" s="36" t="n"/>
+      <c r="Q31" s="36" t="inlineStr"/>
       <c r="R31" s="37" t="n"/>
-      <c r="S31" s="36" t="n"/>
+      <c r="S31" s="36" t="inlineStr"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="39">
         <f>IF(B32="","","REC-"&amp;TEXT(32-8,"000"))</f>
         <v/>
       </c>
-      <c r="B32" s="40" t="n"/>
-      <c r="C32" s="39" t="n"/>
-      <c r="D32" s="40" t="n"/>
-      <c r="E32" s="40" t="n"/>
+      <c r="B32" s="40" t="inlineStr"/>
+      <c r="C32" s="39" t="inlineStr"/>
+      <c r="D32" s="40" t="inlineStr"/>
+      <c r="E32" s="40" t="inlineStr"/>
       <c r="F32" s="41" t="n"/>
       <c r="G32" s="41" t="n"/>
-      <c r="H32" s="39" t="n"/>
+      <c r="H32" s="39" t="inlineStr"/>
       <c r="I32" s="41" t="n"/>
-      <c r="J32" s="40" t="n"/>
+      <c r="J32" s="40" t="inlineStr"/>
       <c r="K32" s="41" t="n"/>
-      <c r="L32" s="39" t="n"/>
+      <c r="L32" s="39" t="inlineStr"/>
       <c r="M32" s="41" t="n"/>
       <c r="N32" s="42" t="n"/>
-      <c r="O32" s="40" t="n"/>
+      <c r="O32" s="40" t="inlineStr"/>
       <c r="P32" s="39">
         <f>IF(B32="","",IF(L32="Yes","LMS Completed (Ready for Exam)",IF(L32="In Progress","LMS In Progress",IF(H32="Yes","ADD Attended - Awaiting LMS",IF(H32="Rescheduled","ADD Rescheduled",IF(H32="Pending","ADD Scheduled",IF(H32="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q32" s="40" t="n"/>
+      <c r="Q32" s="40" t="inlineStr"/>
       <c r="R32" s="41" t="n"/>
-      <c r="S32" s="40" t="n"/>
+      <c r="S32" s="40" t="inlineStr"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="35">
         <f>IF(B33="","","REC-"&amp;TEXT(33-8,"000"))</f>
         <v/>
       </c>
-      <c r="B33" s="36" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="36" t="n"/>
+      <c r="B33" s="36" t="inlineStr"/>
+      <c r="C33" s="35" t="inlineStr"/>
+      <c r="D33" s="36" t="inlineStr"/>
+      <c r="E33" s="36" t="inlineStr"/>
       <c r="F33" s="37" t="n"/>
       <c r="G33" s="37" t="n"/>
-      <c r="H33" s="35" t="n"/>
+      <c r="H33" s="35" t="inlineStr"/>
       <c r="I33" s="37" t="n"/>
-      <c r="J33" s="36" t="n"/>
+      <c r="J33" s="36" t="inlineStr"/>
       <c r="K33" s="37" t="n"/>
-      <c r="L33" s="35" t="n"/>
+      <c r="L33" s="35" t="inlineStr"/>
       <c r="M33" s="37" t="n"/>
       <c r="N33" s="38" t="n"/>
-      <c r="O33" s="36" t="n"/>
+      <c r="O33" s="36" t="inlineStr"/>
       <c r="P33" s="35">
         <f>IF(B33="","",IF(L33="Yes","LMS Completed (Ready for Exam)",IF(L33="In Progress","LMS In Progress",IF(H33="Yes","ADD Attended - Awaiting LMS",IF(H33="Rescheduled","ADD Rescheduled",IF(H33="Pending","ADD Scheduled",IF(H33="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q33" s="36" t="n"/>
+      <c r="Q33" s="36" t="inlineStr"/>
       <c r="R33" s="37" t="n"/>
-      <c r="S33" s="36" t="n"/>
+      <c r="S33" s="36" t="inlineStr"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="39">
         <f>IF(B34="","","REC-"&amp;TEXT(34-8,"000"))</f>
         <v/>
       </c>
-      <c r="B34" s="40" t="n"/>
-      <c r="C34" s="39" t="n"/>
-      <c r="D34" s="40" t="n"/>
-      <c r="E34" s="40" t="n"/>
+      <c r="B34" s="40" t="inlineStr"/>
+      <c r="C34" s="39" t="inlineStr"/>
+      <c r="D34" s="40" t="inlineStr"/>
+      <c r="E34" s="40" t="inlineStr"/>
       <c r="F34" s="41" t="n"/>
       <c r="G34" s="41" t="n"/>
-      <c r="H34" s="39" t="n"/>
+      <c r="H34" s="39" t="inlineStr"/>
       <c r="I34" s="41" t="n"/>
-      <c r="J34" s="40" t="n"/>
+      <c r="J34" s="40" t="inlineStr"/>
       <c r="K34" s="41" t="n"/>
-      <c r="L34" s="39" t="n"/>
+      <c r="L34" s="39" t="inlineStr"/>
       <c r="M34" s="41" t="n"/>
       <c r="N34" s="42" t="n"/>
-      <c r="O34" s="40" t="n"/>
+      <c r="O34" s="40" t="inlineStr"/>
       <c r="P34" s="39">
         <f>IF(B34="","",IF(L34="Yes","LMS Completed (Ready for Exam)",IF(L34="In Progress","LMS In Progress",IF(H34="Yes","ADD Attended - Awaiting LMS",IF(H34="Rescheduled","ADD Rescheduled",IF(H34="Pending","ADD Scheduled",IF(H34="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q34" s="40" t="n"/>
+      <c r="Q34" s="40" t="inlineStr"/>
       <c r="R34" s="41" t="n"/>
-      <c r="S34" s="40" t="n"/>
+      <c r="S34" s="40" t="inlineStr"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="35">
         <f>IF(B35="","","REC-"&amp;TEXT(35-8,"000"))</f>
         <v/>
       </c>
-      <c r="B35" s="36" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="36" t="n"/>
-      <c r="E35" s="36" t="n"/>
+      <c r="B35" s="36" t="inlineStr"/>
+      <c r="C35" s="35" t="inlineStr"/>
+      <c r="D35" s="36" t="inlineStr"/>
+      <c r="E35" s="36" t="inlineStr"/>
       <c r="F35" s="37" t="n"/>
       <c r="G35" s="37" t="n"/>
-      <c r="H35" s="35" t="n"/>
+      <c r="H35" s="35" t="inlineStr"/>
       <c r="I35" s="37" t="n"/>
-      <c r="J35" s="36" t="n"/>
+      <c r="J35" s="36" t="inlineStr"/>
       <c r="K35" s="37" t="n"/>
-      <c r="L35" s="35" t="n"/>
+      <c r="L35" s="35" t="inlineStr"/>
       <c r="M35" s="37" t="n"/>
       <c r="N35" s="38" t="n"/>
-      <c r="O35" s="36" t="n"/>
+      <c r="O35" s="36" t="inlineStr"/>
       <c r="P35" s="35">
         <f>IF(B35="","",IF(L35="Yes","LMS Completed (Ready for Exam)",IF(L35="In Progress","LMS In Progress",IF(H35="Yes","ADD Attended - Awaiting LMS",IF(H35="Rescheduled","ADD Rescheduled",IF(H35="Pending","ADD Scheduled",IF(H35="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q35" s="36" t="n"/>
+      <c r="Q35" s="36" t="inlineStr"/>
       <c r="R35" s="37" t="n"/>
-      <c r="S35" s="36" t="n"/>
+      <c r="S35" s="36" t="inlineStr"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="39">
         <f>IF(B36="","","REC-"&amp;TEXT(36-8,"000"))</f>
         <v/>
       </c>
-      <c r="B36" s="40" t="n"/>
-      <c r="C36" s="39" t="n"/>
-      <c r="D36" s="40" t="n"/>
-      <c r="E36" s="40" t="n"/>
+      <c r="B36" s="40" t="inlineStr"/>
+      <c r="C36" s="39" t="inlineStr"/>
+      <c r="D36" s="40" t="inlineStr"/>
+      <c r="E36" s="40" t="inlineStr"/>
       <c r="F36" s="41" t="n"/>
       <c r="G36" s="41" t="n"/>
-      <c r="H36" s="39" t="n"/>
+      <c r="H36" s="39" t="inlineStr"/>
       <c r="I36" s="41" t="n"/>
-      <c r="J36" s="40" t="n"/>
+      <c r="J36" s="40" t="inlineStr"/>
       <c r="K36" s="41" t="n"/>
-      <c r="L36" s="39" t="n"/>
+      <c r="L36" s="39" t="inlineStr"/>
       <c r="M36" s="41" t="n"/>
       <c r="N36" s="42" t="n"/>
-      <c r="O36" s="40" t="n"/>
+      <c r="O36" s="40" t="inlineStr"/>
       <c r="P36" s="39">
         <f>IF(B36="","",IF(L36="Yes","LMS Completed (Ready for Exam)",IF(L36="In Progress","LMS In Progress",IF(H36="Yes","ADD Attended - Awaiting LMS",IF(H36="Rescheduled","ADD Rescheduled",IF(H36="Pending","ADD Scheduled",IF(H36="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q36" s="40" t="n"/>
+      <c r="Q36" s="40" t="inlineStr"/>
       <c r="R36" s="41" t="n"/>
-      <c r="S36" s="40" t="n"/>
+      <c r="S36" s="40" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="35">
         <f>IF(B37="","","REC-"&amp;TEXT(37-8,"000"))</f>
         <v/>
       </c>
-      <c r="B37" s="36" t="n"/>
-      <c r="C37" s="35" t="n"/>
-      <c r="D37" s="36" t="n"/>
-      <c r="E37" s="36" t="n"/>
+      <c r="B37" s="36" t="inlineStr"/>
+      <c r="C37" s="35" t="inlineStr"/>
+      <c r="D37" s="36" t="inlineStr"/>
+      <c r="E37" s="36" t="inlineStr"/>
       <c r="F37" s="37" t="n"/>
       <c r="G37" s="37" t="n"/>
-      <c r="H37" s="35" t="n"/>
+      <c r="H37" s="35" t="inlineStr"/>
       <c r="I37" s="37" t="n"/>
-      <c r="J37" s="36" t="n"/>
+      <c r="J37" s="36" t="inlineStr"/>
       <c r="K37" s="37" t="n"/>
-      <c r="L37" s="35" t="n"/>
+      <c r="L37" s="35" t="inlineStr"/>
       <c r="M37" s="37" t="n"/>
       <c r="N37" s="38" t="n"/>
-      <c r="O37" s="36" t="n"/>
+      <c r="O37" s="36" t="inlineStr"/>
       <c r="P37" s="35">
         <f>IF(B37="","",IF(L37="Yes","LMS Completed (Ready for Exam)",IF(L37="In Progress","LMS In Progress",IF(H37="Yes","ADD Attended - Awaiting LMS",IF(H37="Rescheduled","ADD Rescheduled",IF(H37="Pending","ADD Scheduled",IF(H37="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q37" s="36" t="n"/>
+      <c r="Q37" s="36" t="inlineStr"/>
       <c r="R37" s="37" t="n"/>
-      <c r="S37" s="36" t="n"/>
+      <c r="S37" s="36" t="inlineStr"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="39">
         <f>IF(B38="","","REC-"&amp;TEXT(38-8,"000"))</f>
         <v/>
       </c>
-      <c r="B38" s="40" t="n"/>
-      <c r="C38" s="39" t="n"/>
-      <c r="D38" s="40" t="n"/>
-      <c r="E38" s="40" t="n"/>
+      <c r="B38" s="40" t="inlineStr"/>
+      <c r="C38" s="39" t="inlineStr"/>
+      <c r="D38" s="40" t="inlineStr"/>
+      <c r="E38" s="40" t="inlineStr"/>
       <c r="F38" s="41" t="n"/>
       <c r="G38" s="41" t="n"/>
-      <c r="H38" s="39" t="n"/>
+      <c r="H38" s="39" t="inlineStr"/>
       <c r="I38" s="41" t="n"/>
-      <c r="J38" s="40" t="n"/>
+      <c r="J38" s="40" t="inlineStr"/>
       <c r="K38" s="41" t="n"/>
-      <c r="L38" s="39" t="n"/>
+      <c r="L38" s="39" t="inlineStr"/>
       <c r="M38" s="41" t="n"/>
       <c r="N38" s="42" t="n"/>
-      <c r="O38" s="40" t="n"/>
+      <c r="O38" s="40" t="inlineStr"/>
       <c r="P38" s="39">
         <f>IF(B38="","",IF(L38="Yes","LMS Completed (Ready for Exam)",IF(L38="In Progress","LMS In Progress",IF(H38="Yes","ADD Attended - Awaiting LMS",IF(H38="Rescheduled","ADD Rescheduled",IF(H38="Pending","ADD Scheduled",IF(H38="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q38" s="40" t="n"/>
+      <c r="Q38" s="40" t="inlineStr"/>
       <c r="R38" s="41" t="n"/>
-      <c r="S38" s="40" t="n"/>
+      <c r="S38" s="40" t="inlineStr"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="35">
         <f>IF(B39="","","REC-"&amp;TEXT(39-8,"000"))</f>
         <v/>
       </c>
-      <c r="B39" s="36" t="n"/>
-      <c r="C39" s="35" t="n"/>
-      <c r="D39" s="36" t="n"/>
-      <c r="E39" s="36" t="n"/>
+      <c r="B39" s="36" t="inlineStr"/>
+      <c r="C39" s="35" t="inlineStr"/>
+      <c r="D39" s="36" t="inlineStr"/>
+      <c r="E39" s="36" t="inlineStr"/>
       <c r="F39" s="37" t="n"/>
       <c r="G39" s="37" t="n"/>
-      <c r="H39" s="35" t="n"/>
+      <c r="H39" s="35" t="inlineStr"/>
       <c r="I39" s="37" t="n"/>
-      <c r="J39" s="36" t="n"/>
+      <c r="J39" s="36" t="inlineStr"/>
       <c r="K39" s="37" t="n"/>
-      <c r="L39" s="35" t="n"/>
+      <c r="L39" s="35" t="inlineStr"/>
       <c r="M39" s="37" t="n"/>
       <c r="N39" s="38" t="n"/>
-      <c r="O39" s="36" t="n"/>
+      <c r="O39" s="36" t="inlineStr"/>
       <c r="P39" s="35">
         <f>IF(B39="","",IF(L39="Yes","LMS Completed (Ready for Exam)",IF(L39="In Progress","LMS In Progress",IF(H39="Yes","ADD Attended - Awaiting LMS",IF(H39="Rescheduled","ADD Rescheduled",IF(H39="Pending","ADD Scheduled",IF(H39="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q39" s="36" t="n"/>
+      <c r="Q39" s="36" t="inlineStr"/>
       <c r="R39" s="37" t="n"/>
-      <c r="S39" s="36" t="n"/>
+      <c r="S39" s="36" t="inlineStr"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="39">
         <f>IF(B40="","","REC-"&amp;TEXT(40-8,"000"))</f>
         <v/>
       </c>
-      <c r="B40" s="40" t="n"/>
-      <c r="C40" s="39" t="n"/>
-      <c r="D40" s="40" t="n"/>
-      <c r="E40" s="40" t="n"/>
+      <c r="B40" s="40" t="inlineStr"/>
+      <c r="C40" s="39" t="inlineStr"/>
+      <c r="D40" s="40" t="inlineStr"/>
+      <c r="E40" s="40" t="inlineStr"/>
       <c r="F40" s="41" t="n"/>
       <c r="G40" s="41" t="n"/>
-      <c r="H40" s="39" t="n"/>
+      <c r="H40" s="39" t="inlineStr"/>
       <c r="I40" s="41" t="n"/>
-      <c r="J40" s="40" t="n"/>
+      <c r="J40" s="40" t="inlineStr"/>
       <c r="K40" s="41" t="n"/>
-      <c r="L40" s="39" t="n"/>
+      <c r="L40" s="39" t="inlineStr"/>
       <c r="M40" s="41" t="n"/>
       <c r="N40" s="42" t="n"/>
-      <c r="O40" s="40" t="n"/>
+      <c r="O40" s="40" t="inlineStr"/>
       <c r="P40" s="39">
         <f>IF(B40="","",IF(L40="Yes","LMS Completed (Ready for Exam)",IF(L40="In Progress","LMS In Progress",IF(H40="Yes","ADD Attended - Awaiting LMS",IF(H40="Rescheduled","ADD Rescheduled",IF(H40="Pending","ADD Scheduled",IF(H40="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q40" s="40" t="n"/>
+      <c r="Q40" s="40" t="inlineStr"/>
       <c r="R40" s="41" t="n"/>
-      <c r="S40" s="40" t="n"/>
+      <c r="S40" s="40" t="inlineStr"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="35">
         <f>IF(B41="","","REC-"&amp;TEXT(41-8,"000"))</f>
         <v/>
       </c>
-      <c r="B41" s="36" t="n"/>
-      <c r="C41" s="35" t="n"/>
-      <c r="D41" s="36" t="n"/>
-      <c r="E41" s="36" t="n"/>
+      <c r="B41" s="36" t="inlineStr"/>
+      <c r="C41" s="35" t="inlineStr"/>
+      <c r="D41" s="36" t="inlineStr"/>
+      <c r="E41" s="36" t="inlineStr"/>
       <c r="F41" s="37" t="n"/>
       <c r="G41" s="37" t="n"/>
-      <c r="H41" s="35" t="n"/>
+      <c r="H41" s="35" t="inlineStr"/>
       <c r="I41" s="37" t="n"/>
-      <c r="J41" s="36" t="n"/>
+      <c r="J41" s="36" t="inlineStr"/>
       <c r="K41" s="37" t="n"/>
-      <c r="L41" s="35" t="n"/>
+      <c r="L41" s="35" t="inlineStr"/>
       <c r="M41" s="37" t="n"/>
       <c r="N41" s="38" t="n"/>
-      <c r="O41" s="36" t="n"/>
+      <c r="O41" s="36" t="inlineStr"/>
       <c r="P41" s="35">
         <f>IF(B41="","",IF(L41="Yes","LMS Completed (Ready for Exam)",IF(L41="In Progress","LMS In Progress",IF(H41="Yes","ADD Attended - Awaiting LMS",IF(H41="Rescheduled","ADD Rescheduled",IF(H41="Pending","ADD Scheduled",IF(H41="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q41" s="36" t="n"/>
+      <c r="Q41" s="36" t="inlineStr"/>
       <c r="R41" s="37" t="n"/>
-      <c r="S41" s="36" t="n"/>
+      <c r="S41" s="36" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="39">
         <f>IF(B42="","","REC-"&amp;TEXT(42-8,"000"))</f>
         <v/>
       </c>
-      <c r="B42" s="40" t="n"/>
-      <c r="C42" s="39" t="n"/>
-      <c r="D42" s="40" t="n"/>
-      <c r="E42" s="40" t="n"/>
+      <c r="B42" s="40" t="inlineStr"/>
+      <c r="C42" s="39" t="inlineStr"/>
+      <c r="D42" s="40" t="inlineStr"/>
+      <c r="E42" s="40" t="inlineStr"/>
       <c r="F42" s="41" t="n"/>
       <c r="G42" s="41" t="n"/>
-      <c r="H42" s="39" t="n"/>
+      <c r="H42" s="39" t="inlineStr"/>
       <c r="I42" s="41" t="n"/>
-      <c r="J42" s="40" t="n"/>
+      <c r="J42" s="40" t="inlineStr"/>
       <c r="K42" s="41" t="n"/>
-      <c r="L42" s="39" t="n"/>
+      <c r="L42" s="39" t="inlineStr"/>
       <c r="M42" s="41" t="n"/>
       <c r="N42" s="42" t="n"/>
-      <c r="O42" s="40" t="n"/>
+      <c r="O42" s="40" t="inlineStr"/>
       <c r="P42" s="39">
         <f>IF(B42="","",IF(L42="Yes","LMS Completed (Ready for Exam)",IF(L42="In Progress","LMS In Progress",IF(H42="Yes","ADD Attended - Awaiting LMS",IF(H42="Rescheduled","ADD Rescheduled",IF(H42="Pending","ADD Scheduled",IF(H42="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q42" s="40" t="n"/>
+      <c r="Q42" s="40" t="inlineStr"/>
       <c r="R42" s="41" t="n"/>
-      <c r="S42" s="40" t="n"/>
+      <c r="S42" s="40" t="inlineStr"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="35">
         <f>IF(B43="","","REC-"&amp;TEXT(43-8,"000"))</f>
         <v/>
       </c>
-      <c r="B43" s="36" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="36" t="n"/>
+      <c r="B43" s="36" t="inlineStr"/>
+      <c r="C43" s="35" t="inlineStr"/>
+      <c r="D43" s="36" t="inlineStr"/>
+      <c r="E43" s="36" t="inlineStr"/>
       <c r="F43" s="37" t="n"/>
       <c r="G43" s="37" t="n"/>
-      <c r="H43" s="35" t="n"/>
+      <c r="H43" s="35" t="inlineStr"/>
       <c r="I43" s="37" t="n"/>
-      <c r="J43" s="36" t="n"/>
+      <c r="J43" s="36" t="inlineStr"/>
       <c r="K43" s="37" t="n"/>
-      <c r="L43" s="35" t="n"/>
+      <c r="L43" s="35" t="inlineStr"/>
       <c r="M43" s="37" t="n"/>
       <c r="N43" s="38" t="n"/>
-      <c r="O43" s="36" t="n"/>
+      <c r="O43" s="36" t="inlineStr"/>
       <c r="P43" s="35">
         <f>IF(B43="","",IF(L43="Yes","LMS Completed (Ready for Exam)",IF(L43="In Progress","LMS In Progress",IF(H43="Yes","ADD Attended - Awaiting LMS",IF(H43="Rescheduled","ADD Rescheduled",IF(H43="Pending","ADD Scheduled",IF(H43="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q43" s="36" t="n"/>
+      <c r="Q43" s="36" t="inlineStr"/>
       <c r="R43" s="37" t="n"/>
-      <c r="S43" s="36" t="n"/>
+      <c r="S43" s="36" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="39">
         <f>IF(B44="","","REC-"&amp;TEXT(44-8,"000"))</f>
         <v/>
       </c>
-      <c r="B44" s="40" t="n"/>
-      <c r="C44" s="39" t="n"/>
-      <c r="D44" s="40" t="n"/>
-      <c r="E44" s="40" t="n"/>
+      <c r="B44" s="40" t="inlineStr"/>
+      <c r="C44" s="39" t="inlineStr"/>
+      <c r="D44" s="40" t="inlineStr"/>
+      <c r="E44" s="40" t="inlineStr"/>
       <c r="F44" s="41" t="n"/>
       <c r="G44" s="41" t="n"/>
-      <c r="H44" s="39" t="n"/>
+      <c r="H44" s="39" t="inlineStr"/>
       <c r="I44" s="41" t="n"/>
-      <c r="J44" s="40" t="n"/>
+      <c r="J44" s="40" t="inlineStr"/>
       <c r="K44" s="41" t="n"/>
-      <c r="L44" s="39" t="n"/>
+      <c r="L44" s="39" t="inlineStr"/>
       <c r="M44" s="41" t="n"/>
       <c r="N44" s="42" t="n"/>
-      <c r="O44" s="40" t="n"/>
+      <c r="O44" s="40" t="inlineStr"/>
       <c r="P44" s="39">
         <f>IF(B44="","",IF(L44="Yes","LMS Completed (Ready for Exam)",IF(L44="In Progress","LMS In Progress",IF(H44="Yes","ADD Attended - Awaiting LMS",IF(H44="Rescheduled","ADD Rescheduled",IF(H44="Pending","ADD Scheduled",IF(H44="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q44" s="40" t="n"/>
+      <c r="Q44" s="40" t="inlineStr"/>
       <c r="R44" s="41" t="n"/>
-      <c r="S44" s="40" t="n"/>
+      <c r="S44" s="40" t="inlineStr"/>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="35">
         <f>IF(B45="","","REC-"&amp;TEXT(45-8,"000"))</f>
         <v/>
       </c>
-      <c r="B45" s="36" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="36" t="n"/>
-      <c r="E45" s="36" t="n"/>
+      <c r="B45" s="36" t="inlineStr"/>
+      <c r="C45" s="35" t="inlineStr"/>
+      <c r="D45" s="36" t="inlineStr"/>
+      <c r="E45" s="36" t="inlineStr"/>
       <c r="F45" s="37" t="n"/>
       <c r="G45" s="37" t="n"/>
-      <c r="H45" s="35" t="n"/>
+      <c r="H45" s="35" t="inlineStr"/>
       <c r="I45" s="37" t="n"/>
-      <c r="J45" s="36" t="n"/>
+      <c r="J45" s="36" t="inlineStr"/>
       <c r="K45" s="37" t="n"/>
-      <c r="L45" s="35" t="n"/>
+      <c r="L45" s="35" t="inlineStr"/>
       <c r="M45" s="37" t="n"/>
       <c r="N45" s="38" t="n"/>
-      <c r="O45" s="36" t="n"/>
+      <c r="O45" s="36" t="inlineStr"/>
       <c r="P45" s="35">
         <f>IF(B45="","",IF(L45="Yes","LMS Completed (Ready for Exam)",IF(L45="In Progress","LMS In Progress",IF(H45="Yes","ADD Attended - Awaiting LMS",IF(H45="Rescheduled","ADD Rescheduled",IF(H45="Pending","ADD Scheduled",IF(H45="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q45" s="36" t="n"/>
+      <c r="Q45" s="36" t="inlineStr"/>
       <c r="R45" s="37" t="n"/>
-      <c r="S45" s="36" t="n"/>
+      <c r="S45" s="36" t="inlineStr"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="39">
         <f>IF(B46="","","REC-"&amp;TEXT(46-8,"000"))</f>
         <v/>
       </c>
-      <c r="B46" s="40" t="n"/>
-      <c r="C46" s="39" t="n"/>
-      <c r="D46" s="40" t="n"/>
-      <c r="E46" s="40" t="n"/>
+      <c r="B46" s="40" t="inlineStr"/>
+      <c r="C46" s="39" t="inlineStr"/>
+      <c r="D46" s="40" t="inlineStr"/>
+      <c r="E46" s="40" t="inlineStr"/>
       <c r="F46" s="41" t="n"/>
       <c r="G46" s="41" t="n"/>
-      <c r="H46" s="39" t="n"/>
+      <c r="H46" s="39" t="inlineStr"/>
       <c r="I46" s="41" t="n"/>
-      <c r="J46" s="40" t="n"/>
+      <c r="J46" s="40" t="inlineStr"/>
       <c r="K46" s="41" t="n"/>
-      <c r="L46" s="39" t="n"/>
+      <c r="L46" s="39" t="inlineStr"/>
       <c r="M46" s="41" t="n"/>
       <c r="N46" s="42" t="n"/>
-      <c r="O46" s="40" t="n"/>
+      <c r="O46" s="40" t="inlineStr"/>
       <c r="P46" s="39">
         <f>IF(B46="","",IF(L46="Yes","LMS Completed (Ready for Exam)",IF(L46="In Progress","LMS In Progress",IF(H46="Yes","ADD Attended - Awaiting LMS",IF(H46="Rescheduled","ADD Rescheduled",IF(H46="Pending","ADD Scheduled",IF(H46="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q46" s="40" t="n"/>
+      <c r="Q46" s="40" t="inlineStr"/>
       <c r="R46" s="41" t="n"/>
-      <c r="S46" s="40" t="n"/>
+      <c r="S46" s="40" t="inlineStr"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="35">
         <f>IF(B47="","","REC-"&amp;TEXT(47-8,"000"))</f>
         <v/>
       </c>
-      <c r="B47" s="36" t="n"/>
-      <c r="C47" s="35" t="n"/>
-      <c r="D47" s="36" t="n"/>
-      <c r="E47" s="36" t="n"/>
+      <c r="B47" s="36" t="inlineStr"/>
+      <c r="C47" s="35" t="inlineStr"/>
+      <c r="D47" s="36" t="inlineStr"/>
+      <c r="E47" s="36" t="inlineStr"/>
       <c r="F47" s="37" t="n"/>
       <c r="G47" s="37" t="n"/>
-      <c r="H47" s="35" t="n"/>
+      <c r="H47" s="35" t="inlineStr"/>
       <c r="I47" s="37" t="n"/>
-      <c r="J47" s="36" t="n"/>
+      <c r="J47" s="36" t="inlineStr"/>
       <c r="K47" s="37" t="n"/>
-      <c r="L47" s="35" t="n"/>
+      <c r="L47" s="35" t="inlineStr"/>
       <c r="M47" s="37" t="n"/>
       <c r="N47" s="38" t="n"/>
-      <c r="O47" s="36" t="n"/>
+      <c r="O47" s="36" t="inlineStr"/>
       <c r="P47" s="35">
         <f>IF(B47="","",IF(L47="Yes","LMS Completed (Ready for Exam)",IF(L47="In Progress","LMS In Progress",IF(H47="Yes","ADD Attended - Awaiting LMS",IF(H47="Rescheduled","ADD Rescheduled",IF(H47="Pending","ADD Scheduled",IF(H47="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q47" s="36" t="n"/>
+      <c r="Q47" s="36" t="inlineStr"/>
       <c r="R47" s="37" t="n"/>
-      <c r="S47" s="36" t="n"/>
+      <c r="S47" s="36" t="inlineStr"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="39">
         <f>IF(B48="","","REC-"&amp;TEXT(48-8,"000"))</f>
         <v/>
       </c>
-      <c r="B48" s="40" t="n"/>
-      <c r="C48" s="39" t="n"/>
-      <c r="D48" s="40" t="n"/>
-      <c r="E48" s="40" t="n"/>
+      <c r="B48" s="40" t="inlineStr"/>
+      <c r="C48" s="39" t="inlineStr"/>
+      <c r="D48" s="40" t="inlineStr"/>
+      <c r="E48" s="40" t="inlineStr"/>
       <c r="F48" s="41" t="n"/>
       <c r="G48" s="41" t="n"/>
-      <c r="H48" s="39" t="n"/>
+      <c r="H48" s="39" t="inlineStr"/>
       <c r="I48" s="41" t="n"/>
-      <c r="J48" s="40" t="n"/>
+      <c r="J48" s="40" t="inlineStr"/>
       <c r="K48" s="41" t="n"/>
-      <c r="L48" s="39" t="n"/>
+      <c r="L48" s="39" t="inlineStr"/>
       <c r="M48" s="41" t="n"/>
       <c r="N48" s="42" t="n"/>
-      <c r="O48" s="40" t="n"/>
+      <c r="O48" s="40" t="inlineStr"/>
       <c r="P48" s="39">
         <f>IF(B48="","",IF(L48="Yes","LMS Completed (Ready for Exam)",IF(L48="In Progress","LMS In Progress",IF(H48="Yes","ADD Attended - Awaiting LMS",IF(H48="Rescheduled","ADD Rescheduled",IF(H48="Pending","ADD Scheduled",IF(H48="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q48" s="40" t="n"/>
+      <c r="Q48" s="40" t="inlineStr"/>
       <c r="R48" s="41" t="n"/>
-      <c r="S48" s="40" t="n"/>
+      <c r="S48" s="40" t="inlineStr"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="35">
         <f>IF(B49="","","REC-"&amp;TEXT(49-8,"000"))</f>
         <v/>
       </c>
-      <c r="B49" s="36" t="n"/>
-      <c r="C49" s="35" t="n"/>
-      <c r="D49" s="36" t="n"/>
-      <c r="E49" s="36" t="n"/>
+      <c r="B49" s="36" t="inlineStr"/>
+      <c r="C49" s="35" t="inlineStr"/>
+      <c r="D49" s="36" t="inlineStr"/>
+      <c r="E49" s="36" t="inlineStr"/>
       <c r="F49" s="37" t="n"/>
       <c r="G49" s="37" t="n"/>
-      <c r="H49" s="35" t="n"/>
+      <c r="H49" s="35" t="inlineStr"/>
       <c r="I49" s="37" t="n"/>
-      <c r="J49" s="36" t="n"/>
+      <c r="J49" s="36" t="inlineStr"/>
       <c r="K49" s="37" t="n"/>
-      <c r="L49" s="35" t="n"/>
+      <c r="L49" s="35" t="inlineStr"/>
       <c r="M49" s="37" t="n"/>
       <c r="N49" s="38" t="n"/>
-      <c r="O49" s="36" t="n"/>
+      <c r="O49" s="36" t="inlineStr"/>
       <c r="P49" s="35">
         <f>IF(B49="","",IF(L49="Yes","LMS Completed (Ready for Exam)",IF(L49="In Progress","LMS In Progress",IF(H49="Yes","ADD Attended - Awaiting LMS",IF(H49="Rescheduled","ADD Rescheduled",IF(H49="Pending","ADD Scheduled",IF(H49="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q49" s="36" t="n"/>
+      <c r="Q49" s="36" t="inlineStr"/>
       <c r="R49" s="37" t="n"/>
-      <c r="S49" s="36" t="n"/>
+      <c r="S49" s="36" t="inlineStr"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="39">
         <f>IF(B50="","","REC-"&amp;TEXT(50-8,"000"))</f>
         <v/>
       </c>
-      <c r="B50" s="40" t="n"/>
-      <c r="C50" s="39" t="n"/>
-      <c r="D50" s="40" t="n"/>
-      <c r="E50" s="40" t="n"/>
+      <c r="B50" s="40" t="inlineStr"/>
+      <c r="C50" s="39" t="inlineStr"/>
+      <c r="D50" s="40" t="inlineStr"/>
+      <c r="E50" s="40" t="inlineStr"/>
       <c r="F50" s="41" t="n"/>
       <c r="G50" s="41" t="n"/>
-      <c r="H50" s="39" t="n"/>
+      <c r="H50" s="39" t="inlineStr"/>
       <c r="I50" s="41" t="n"/>
-      <c r="J50" s="40" t="n"/>
+      <c r="J50" s="40" t="inlineStr"/>
       <c r="K50" s="41" t="n"/>
-      <c r="L50" s="39" t="n"/>
+      <c r="L50" s="39" t="inlineStr"/>
       <c r="M50" s="41" t="n"/>
       <c r="N50" s="42" t="n"/>
-      <c r="O50" s="40" t="n"/>
+      <c r="O50" s="40" t="inlineStr"/>
       <c r="P50" s="39">
         <f>IF(B50="","",IF(L50="Yes","LMS Completed (Ready for Exam)",IF(L50="In Progress","LMS In Progress",IF(H50="Yes","ADD Attended - Awaiting LMS",IF(H50="Rescheduled","ADD Rescheduled",IF(H50="Pending","ADD Scheduled",IF(H50="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q50" s="40" t="n"/>
+      <c r="Q50" s="40" t="inlineStr"/>
       <c r="R50" s="41" t="n"/>
-      <c r="S50" s="40" t="n"/>
+      <c r="S50" s="40" t="inlineStr"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="35">
         <f>IF(B51="","","REC-"&amp;TEXT(51-8,"000"))</f>
         <v/>
       </c>
-      <c r="B51" s="36" t="n"/>
-      <c r="C51" s="35" t="n"/>
-      <c r="D51" s="36" t="n"/>
-      <c r="E51" s="36" t="n"/>
+      <c r="B51" s="36" t="inlineStr"/>
+      <c r="C51" s="35" t="inlineStr"/>
+      <c r="D51" s="36" t="inlineStr"/>
+      <c r="E51" s="36" t="inlineStr"/>
       <c r="F51" s="37" t="n"/>
       <c r="G51" s="37" t="n"/>
-      <c r="H51" s="35" t="n"/>
+      <c r="H51" s="35" t="inlineStr"/>
       <c r="I51" s="37" t="n"/>
-      <c r="J51" s="36" t="n"/>
+      <c r="J51" s="36" t="inlineStr"/>
       <c r="K51" s="37" t="n"/>
-      <c r="L51" s="35" t="n"/>
+      <c r="L51" s="35" t="inlineStr"/>
       <c r="M51" s="37" t="n"/>
       <c r="N51" s="38" t="n"/>
-      <c r="O51" s="36" t="n"/>
+      <c r="O51" s="36" t="inlineStr"/>
       <c r="P51" s="35">
         <f>IF(B51="","",IF(L51="Yes","LMS Completed (Ready for Exam)",IF(L51="In Progress","LMS In Progress",IF(H51="Yes","ADD Attended - Awaiting LMS",IF(H51="Rescheduled","ADD Rescheduled",IF(H51="Pending","ADD Scheduled",IF(H51="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q51" s="36" t="n"/>
+      <c r="Q51" s="36" t="inlineStr"/>
       <c r="R51" s="37" t="n"/>
-      <c r="S51" s="36" t="n"/>
+      <c r="S51" s="36" t="inlineStr"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="39">
         <f>IF(B52="","","REC-"&amp;TEXT(52-8,"000"))</f>
         <v/>
       </c>
-      <c r="B52" s="40" t="n"/>
-      <c r="C52" s="39" t="n"/>
-      <c r="D52" s="40" t="n"/>
-      <c r="E52" s="40" t="n"/>
+      <c r="B52" s="40" t="inlineStr"/>
+      <c r="C52" s="39" t="inlineStr"/>
+      <c r="D52" s="40" t="inlineStr"/>
+      <c r="E52" s="40" t="inlineStr"/>
       <c r="F52" s="41" t="n"/>
       <c r="G52" s="41" t="n"/>
-      <c r="H52" s="39" t="n"/>
+      <c r="H52" s="39" t="inlineStr"/>
       <c r="I52" s="41" t="n"/>
-      <c r="J52" s="40" t="n"/>
+      <c r="J52" s="40" t="inlineStr"/>
       <c r="K52" s="41" t="n"/>
-      <c r="L52" s="39" t="n"/>
+      <c r="L52" s="39" t="inlineStr"/>
       <c r="M52" s="41" t="n"/>
       <c r="N52" s="42" t="n"/>
-      <c r="O52" s="40" t="n"/>
+      <c r="O52" s="40" t="inlineStr"/>
       <c r="P52" s="39">
         <f>IF(B52="","",IF(L52="Yes","LMS Completed (Ready for Exam)",IF(L52="In Progress","LMS In Progress",IF(H52="Yes","ADD Attended - Awaiting LMS",IF(H52="Rescheduled","ADD Rescheduled",IF(H52="Pending","ADD Scheduled",IF(H52="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q52" s="40" t="n"/>
+      <c r="Q52" s="40" t="inlineStr"/>
       <c r="R52" s="41" t="n"/>
-      <c r="S52" s="40" t="n"/>
+      <c r="S52" s="40" t="inlineStr"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="35">
         <f>IF(B53="","","REC-"&amp;TEXT(53-8,"000"))</f>
         <v/>
       </c>
-      <c r="B53" s="36" t="n"/>
-      <c r="C53" s="35" t="n"/>
-      <c r="D53" s="36" t="n"/>
-      <c r="E53" s="36" t="n"/>
+      <c r="B53" s="36" t="inlineStr"/>
+      <c r="C53" s="35" t="inlineStr"/>
+      <c r="D53" s="36" t="inlineStr"/>
+      <c r="E53" s="36" t="inlineStr"/>
       <c r="F53" s="37" t="n"/>
       <c r="G53" s="37" t="n"/>
-      <c r="H53" s="35" t="n"/>
+      <c r="H53" s="35" t="inlineStr"/>
       <c r="I53" s="37" t="n"/>
-      <c r="J53" s="36" t="n"/>
+      <c r="J53" s="36" t="inlineStr"/>
       <c r="K53" s="37" t="n"/>
-      <c r="L53" s="35" t="n"/>
+      <c r="L53" s="35" t="inlineStr"/>
       <c r="M53" s="37" t="n"/>
       <c r="N53" s="38" t="n"/>
-      <c r="O53" s="36" t="n"/>
+      <c r="O53" s="36" t="inlineStr"/>
       <c r="P53" s="35">
         <f>IF(B53="","",IF(L53="Yes","LMS Completed (Ready for Exam)",IF(L53="In Progress","LMS In Progress",IF(H53="Yes","ADD Attended - Awaiting LMS",IF(H53="Rescheduled","ADD Rescheduled",IF(H53="Pending","ADD Scheduled",IF(H53="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q53" s="36" t="n"/>
+      <c r="Q53" s="36" t="inlineStr"/>
       <c r="R53" s="37" t="n"/>
-      <c r="S53" s="36" t="n"/>
+      <c r="S53" s="36" t="inlineStr"/>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="39">
         <f>IF(B54="","","REC-"&amp;TEXT(54-8,"000"))</f>
         <v/>
       </c>
-      <c r="B54" s="40" t="n"/>
-      <c r="C54" s="39" t="n"/>
-      <c r="D54" s="40" t="n"/>
-      <c r="E54" s="40" t="n"/>
+      <c r="B54" s="40" t="inlineStr"/>
+      <c r="C54" s="39" t="inlineStr"/>
+      <c r="D54" s="40" t="inlineStr"/>
+      <c r="E54" s="40" t="inlineStr"/>
       <c r="F54" s="41" t="n"/>
       <c r="G54" s="41" t="n"/>
-      <c r="H54" s="39" t="n"/>
+      <c r="H54" s="39" t="inlineStr"/>
       <c r="I54" s="41" t="n"/>
-      <c r="J54" s="40" t="n"/>
+      <c r="J54" s="40" t="inlineStr"/>
       <c r="K54" s="41" t="n"/>
-      <c r="L54" s="39" t="n"/>
+      <c r="L54" s="39" t="inlineStr"/>
       <c r="M54" s="41" t="n"/>
       <c r="N54" s="42" t="n"/>
-      <c r="O54" s="40" t="n"/>
+      <c r="O54" s="40" t="inlineStr"/>
       <c r="P54" s="39">
         <f>IF(B54="","",IF(L54="Yes","LMS Completed (Ready for Exam)",IF(L54="In Progress","LMS In Progress",IF(H54="Yes","ADD Attended - Awaiting LMS",IF(H54="Rescheduled","ADD Rescheduled",IF(H54="Pending","ADD Scheduled",IF(H54="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q54" s="40" t="n"/>
+      <c r="Q54" s="40" t="inlineStr"/>
       <c r="R54" s="41" t="n"/>
-      <c r="S54" s="40" t="n"/>
+      <c r="S54" s="40" t="inlineStr"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="35">
         <f>IF(B55="","","REC-"&amp;TEXT(55-8,"000"))</f>
         <v/>
       </c>
-      <c r="B55" s="36" t="n"/>
-      <c r="C55" s="35" t="n"/>
-      <c r="D55" s="36" t="n"/>
-      <c r="E55" s="36" t="n"/>
+      <c r="B55" s="36" t="inlineStr"/>
+      <c r="C55" s="35" t="inlineStr"/>
+      <c r="D55" s="36" t="inlineStr"/>
+      <c r="E55" s="36" t="inlineStr"/>
       <c r="F55" s="37" t="n"/>
       <c r="G55" s="37" t="n"/>
-      <c r="H55" s="35" t="n"/>
+      <c r="H55" s="35" t="inlineStr"/>
       <c r="I55" s="37" t="n"/>
-      <c r="J55" s="36" t="n"/>
+      <c r="J55" s="36" t="inlineStr"/>
       <c r="K55" s="37" t="n"/>
-      <c r="L55" s="35" t="n"/>
+      <c r="L55" s="35" t="inlineStr"/>
       <c r="M55" s="37" t="n"/>
       <c r="N55" s="38" t="n"/>
-      <c r="O55" s="36" t="n"/>
+      <c r="O55" s="36" t="inlineStr"/>
       <c r="P55" s="35">
         <f>IF(B55="","",IF(L55="Yes","LMS Completed (Ready for Exam)",IF(L55="In Progress","LMS In Progress",IF(H55="Yes","ADD Attended - Awaiting LMS",IF(H55="Rescheduled","ADD Rescheduled",IF(H55="Pending","ADD Scheduled",IF(H55="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q55" s="36" t="n"/>
+      <c r="Q55" s="36" t="inlineStr"/>
       <c r="R55" s="37" t="n"/>
-      <c r="S55" s="36" t="n"/>
+      <c r="S55" s="36" t="inlineStr"/>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="39">
         <f>IF(B56="","","REC-"&amp;TEXT(56-8,"000"))</f>
         <v/>
       </c>
-      <c r="B56" s="40" t="n"/>
-      <c r="C56" s="39" t="n"/>
-      <c r="D56" s="40" t="n"/>
-      <c r="E56" s="40" t="n"/>
+      <c r="B56" s="40" t="inlineStr"/>
+      <c r="C56" s="39" t="inlineStr"/>
+      <c r="D56" s="40" t="inlineStr"/>
+      <c r="E56" s="40" t="inlineStr"/>
       <c r="F56" s="41" t="n"/>
       <c r="G56" s="41" t="n"/>
-      <c r="H56" s="39" t="n"/>
+      <c r="H56" s="39" t="inlineStr"/>
       <c r="I56" s="41" t="n"/>
-      <c r="J56" s="40" t="n"/>
+      <c r="J56" s="40" t="inlineStr"/>
       <c r="K56" s="41" t="n"/>
-      <c r="L56" s="39" t="n"/>
+      <c r="L56" s="39" t="inlineStr"/>
       <c r="M56" s="41" t="n"/>
       <c r="N56" s="42" t="n"/>
-      <c r="O56" s="40" t="n"/>
+      <c r="O56" s="40" t="inlineStr"/>
       <c r="P56" s="39">
         <f>IF(B56="","",IF(L56="Yes","LMS Completed (Ready for Exam)",IF(L56="In Progress","LMS In Progress",IF(H56="Yes","ADD Attended - Awaiting LMS",IF(H56="Rescheduled","ADD Rescheduled",IF(H56="Pending","ADD Scheduled",IF(H56="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q56" s="40" t="n"/>
+      <c r="Q56" s="40" t="inlineStr"/>
       <c r="R56" s="41" t="n"/>
-      <c r="S56" s="40" t="n"/>
+      <c r="S56" s="40" t="inlineStr"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="35">
         <f>IF(B57="","","REC-"&amp;TEXT(57-8,"000"))</f>
         <v/>
       </c>
-      <c r="B57" s="36" t="n"/>
-      <c r="C57" s="35" t="n"/>
-      <c r="D57" s="36" t="n"/>
-      <c r="E57" s="36" t="n"/>
+      <c r="B57" s="36" t="inlineStr"/>
+      <c r="C57" s="35" t="inlineStr"/>
+      <c r="D57" s="36" t="inlineStr"/>
+      <c r="E57" s="36" t="inlineStr"/>
       <c r="F57" s="37" t="n"/>
       <c r="G57" s="37" t="n"/>
-      <c r="H57" s="35" t="n"/>
+      <c r="H57" s="35" t="inlineStr"/>
       <c r="I57" s="37" t="n"/>
-      <c r="J57" s="36" t="n"/>
+      <c r="J57" s="36" t="inlineStr"/>
       <c r="K57" s="37" t="n"/>
-      <c r="L57" s="35" t="n"/>
+      <c r="L57" s="35" t="inlineStr"/>
       <c r="M57" s="37" t="n"/>
       <c r="N57" s="38" t="n"/>
-      <c r="O57" s="36" t="n"/>
+      <c r="O57" s="36" t="inlineStr"/>
       <c r="P57" s="35">
         <f>IF(B57="","",IF(L57="Yes","LMS Completed (Ready for Exam)",IF(L57="In Progress","LMS In Progress",IF(H57="Yes","ADD Attended - Awaiting LMS",IF(H57="Rescheduled","ADD Rescheduled",IF(H57="Pending","ADD Scheduled",IF(H57="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q57" s="36" t="n"/>
+      <c r="Q57" s="36" t="inlineStr"/>
       <c r="R57" s="37" t="n"/>
-      <c r="S57" s="36" t="n"/>
+      <c r="S57" s="36" t="inlineStr"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="39">
         <f>IF(B58="","","REC-"&amp;TEXT(58-8,"000"))</f>
         <v/>
       </c>
-      <c r="B58" s="40" t="n"/>
-      <c r="C58" s="39" t="n"/>
-      <c r="D58" s="40" t="n"/>
-      <c r="E58" s="40" t="n"/>
+      <c r="B58" s="40" t="inlineStr"/>
+      <c r="C58" s="39" t="inlineStr"/>
+      <c r="D58" s="40" t="inlineStr"/>
+      <c r="E58" s="40" t="inlineStr"/>
       <c r="F58" s="41" t="n"/>
       <c r="G58" s="41" t="n"/>
-      <c r="H58" s="39" t="n"/>
+      <c r="H58" s="39" t="inlineStr"/>
       <c r="I58" s="41" t="n"/>
-      <c r="J58" s="40" t="n"/>
+      <c r="J58" s="40" t="inlineStr"/>
       <c r="K58" s="41" t="n"/>
-      <c r="L58" s="39" t="n"/>
+      <c r="L58" s="39" t="inlineStr"/>
       <c r="M58" s="41" t="n"/>
       <c r="N58" s="42" t="n"/>
-      <c r="O58" s="40" t="n"/>
+      <c r="O58" s="40" t="inlineStr"/>
       <c r="P58" s="39">
         <f>IF(B58="","",IF(L58="Yes","LMS Completed (Ready for Exam)",IF(L58="In Progress","LMS In Progress",IF(H58="Yes","ADD Attended - Awaiting LMS",IF(H58="Rescheduled","ADD Rescheduled",IF(H58="Pending","ADD Scheduled",IF(H58="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q58" s="40" t="n"/>
+      <c r="Q58" s="40" t="inlineStr"/>
       <c r="R58" s="41" t="n"/>
-      <c r="S58" s="40" t="n"/>
+      <c r="S58" s="40" t="inlineStr"/>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="35">
         <f>IF(B59="","","REC-"&amp;TEXT(59-8,"000"))</f>
         <v/>
       </c>
-      <c r="B59" s="36" t="n"/>
-      <c r="C59" s="35" t="n"/>
-      <c r="D59" s="36" t="n"/>
-      <c r="E59" s="36" t="n"/>
+      <c r="B59" s="36" t="inlineStr"/>
+      <c r="C59" s="35" t="inlineStr"/>
+      <c r="D59" s="36" t="inlineStr"/>
+      <c r="E59" s="36" t="inlineStr"/>
       <c r="F59" s="37" t="n"/>
       <c r="G59" s="37" t="n"/>
-      <c r="H59" s="35" t="n"/>
+      <c r="H59" s="35" t="inlineStr"/>
       <c r="I59" s="37" t="n"/>
-      <c r="J59" s="36" t="n"/>
+      <c r="J59" s="36" t="inlineStr"/>
       <c r="K59" s="37" t="n"/>
-      <c r="L59" s="35" t="n"/>
+      <c r="L59" s="35" t="inlineStr"/>
       <c r="M59" s="37" t="n"/>
       <c r="N59" s="38" t="n"/>
-      <c r="O59" s="36" t="n"/>
+      <c r="O59" s="36" t="inlineStr"/>
       <c r="P59" s="35">
         <f>IF(B59="","",IF(L59="Yes","LMS Completed (Ready for Exam)",IF(L59="In Progress","LMS In Progress",IF(H59="Yes","ADD Attended - Awaiting LMS",IF(H59="Rescheduled","ADD Rescheduled",IF(H59="Pending","ADD Scheduled",IF(H59="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q59" s="36" t="n"/>
+      <c r="Q59" s="36" t="inlineStr"/>
       <c r="R59" s="37" t="n"/>
-      <c r="S59" s="36" t="n"/>
+      <c r="S59" s="36" t="inlineStr"/>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="39">
         <f>IF(B60="","","REC-"&amp;TEXT(60-8,"000"))</f>
         <v/>
       </c>
-      <c r="B60" s="40" t="n"/>
-      <c r="C60" s="39" t="n"/>
-      <c r="D60" s="40" t="n"/>
-      <c r="E60" s="40" t="n"/>
+      <c r="B60" s="40" t="inlineStr"/>
+      <c r="C60" s="39" t="inlineStr"/>
+      <c r="D60" s="40" t="inlineStr"/>
+      <c r="E60" s="40" t="inlineStr"/>
       <c r="F60" s="41" t="n"/>
       <c r="G60" s="41" t="n"/>
-      <c r="H60" s="39" t="n"/>
+      <c r="H60" s="39" t="inlineStr"/>
       <c r="I60" s="41" t="n"/>
-      <c r="J60" s="40" t="n"/>
+      <c r="J60" s="40" t="inlineStr"/>
       <c r="K60" s="41" t="n"/>
-      <c r="L60" s="39" t="n"/>
+      <c r="L60" s="39" t="inlineStr"/>
       <c r="M60" s="41" t="n"/>
       <c r="N60" s="42" t="n"/>
-      <c r="O60" s="40" t="n"/>
+      <c r="O60" s="40" t="inlineStr"/>
       <c r="P60" s="39">
         <f>IF(B60="","",IF(L60="Yes","LMS Completed (Ready for Exam)",IF(L60="In Progress","LMS In Progress",IF(H60="Yes","ADD Attended - Awaiting LMS",IF(H60="Rescheduled","ADD Rescheduled",IF(H60="Pending","ADD Scheduled",IF(H60="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q60" s="40" t="n"/>
+      <c r="Q60" s="40" t="inlineStr"/>
       <c r="R60" s="41" t="n"/>
-      <c r="S60" s="40" t="n"/>
+      <c r="S60" s="40" t="inlineStr"/>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="35">
         <f>IF(B61="","","REC-"&amp;TEXT(61-8,"000"))</f>
         <v/>
       </c>
-      <c r="B61" s="36" t="n"/>
-      <c r="C61" s="35" t="n"/>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="36" t="n"/>
+      <c r="B61" s="36" t="inlineStr"/>
+      <c r="C61" s="35" t="inlineStr"/>
+      <c r="D61" s="36" t="inlineStr"/>
+      <c r="E61" s="36" t="inlineStr"/>
       <c r="F61" s="37" t="n"/>
       <c r="G61" s="37" t="n"/>
-      <c r="H61" s="35" t="n"/>
+      <c r="H61" s="35" t="inlineStr"/>
       <c r="I61" s="37" t="n"/>
-      <c r="J61" s="36" t="n"/>
+      <c r="J61" s="36" t="inlineStr"/>
       <c r="K61" s="37" t="n"/>
-      <c r="L61" s="35" t="n"/>
+      <c r="L61" s="35" t="inlineStr"/>
       <c r="M61" s="37" t="n"/>
       <c r="N61" s="38" t="n"/>
-      <c r="O61" s="36" t="n"/>
+      <c r="O61" s="36" t="inlineStr"/>
       <c r="P61" s="35">
         <f>IF(B61="","",IF(L61="Yes","LMS Completed (Ready for Exam)",IF(L61="In Progress","LMS In Progress",IF(H61="Yes","ADD Attended - Awaiting LMS",IF(H61="Rescheduled","ADD Rescheduled",IF(H61="Pending","ADD Scheduled",IF(H61="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q61" s="36" t="n"/>
+      <c r="Q61" s="36" t="inlineStr"/>
       <c r="R61" s="37" t="n"/>
-      <c r="S61" s="36" t="n"/>
+      <c r="S61" s="36" t="inlineStr"/>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="39">
         <f>IF(B62="","","REC-"&amp;TEXT(62-8,"000"))</f>
         <v/>
       </c>
-      <c r="B62" s="40" t="n"/>
-      <c r="C62" s="39" t="n"/>
-      <c r="D62" s="40" t="n"/>
-      <c r="E62" s="40" t="n"/>
+      <c r="B62" s="40" t="inlineStr"/>
+      <c r="C62" s="39" t="inlineStr"/>
+      <c r="D62" s="40" t="inlineStr"/>
+      <c r="E62" s="40" t="inlineStr"/>
       <c r="F62" s="41" t="n"/>
       <c r="G62" s="41" t="n"/>
-      <c r="H62" s="39" t="n"/>
+      <c r="H62" s="39" t="inlineStr"/>
       <c r="I62" s="41" t="n"/>
-      <c r="J62" s="40" t="n"/>
+      <c r="J62" s="40" t="inlineStr"/>
       <c r="K62" s="41" t="n"/>
-      <c r="L62" s="39" t="n"/>
+      <c r="L62" s="39" t="inlineStr"/>
       <c r="M62" s="41" t="n"/>
       <c r="N62" s="42" t="n"/>
-      <c r="O62" s="40" t="n"/>
+      <c r="O62" s="40" t="inlineStr"/>
       <c r="P62" s="39">
         <f>IF(B62="","",IF(L62="Yes","LMS Completed (Ready for Exam)",IF(L62="In Progress","LMS In Progress",IF(H62="Yes","ADD Attended - Awaiting LMS",IF(H62="Rescheduled","ADD Rescheduled",IF(H62="Pending","ADD Scheduled",IF(H62="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q62" s="40" t="n"/>
+      <c r="Q62" s="40" t="inlineStr"/>
       <c r="R62" s="41" t="n"/>
-      <c r="S62" s="40" t="n"/>
+      <c r="S62" s="40" t="inlineStr"/>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="35">
         <f>IF(B63="","","REC-"&amp;TEXT(63-8,"000"))</f>
         <v/>
       </c>
-      <c r="B63" s="36" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="36" t="n"/>
-      <c r="E63" s="36" t="n"/>
+      <c r="B63" s="36" t="inlineStr"/>
+      <c r="C63" s="35" t="inlineStr"/>
+      <c r="D63" s="36" t="inlineStr"/>
+      <c r="E63" s="36" t="inlineStr"/>
       <c r="F63" s="37" t="n"/>
       <c r="G63" s="37" t="n"/>
-      <c r="H63" s="35" t="n"/>
+      <c r="H63" s="35" t="inlineStr"/>
       <c r="I63" s="37" t="n"/>
-      <c r="J63" s="36" t="n"/>
+      <c r="J63" s="36" t="inlineStr"/>
       <c r="K63" s="37" t="n"/>
-      <c r="L63" s="35" t="n"/>
+      <c r="L63" s="35" t="inlineStr"/>
       <c r="M63" s="37" t="n"/>
       <c r="N63" s="38" t="n"/>
-      <c r="O63" s="36" t="n"/>
+      <c r="O63" s="36" t="inlineStr"/>
       <c r="P63" s="35">
         <f>IF(B63="","",IF(L63="Yes","LMS Completed (Ready for Exam)",IF(L63="In Progress","LMS In Progress",IF(H63="Yes","ADD Attended - Awaiting LMS",IF(H63="Rescheduled","ADD Rescheduled",IF(H63="Pending","ADD Scheduled",IF(H63="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q63" s="36" t="n"/>
+      <c r="Q63" s="36" t="inlineStr"/>
       <c r="R63" s="37" t="n"/>
-      <c r="S63" s="36" t="n"/>
+      <c r="S63" s="36" t="inlineStr"/>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="39">
         <f>IF(B64="","","REC-"&amp;TEXT(64-8,"000"))</f>
         <v/>
       </c>
-      <c r="B64" s="40" t="n"/>
-      <c r="C64" s="39" t="n"/>
-      <c r="D64" s="40" t="n"/>
-      <c r="E64" s="40" t="n"/>
+      <c r="B64" s="40" t="inlineStr"/>
+      <c r="C64" s="39" t="inlineStr"/>
+      <c r="D64" s="40" t="inlineStr"/>
+      <c r="E64" s="40" t="inlineStr"/>
       <c r="F64" s="41" t="n"/>
       <c r="G64" s="41" t="n"/>
-      <c r="H64" s="39" t="n"/>
+      <c r="H64" s="39" t="inlineStr"/>
       <c r="I64" s="41" t="n"/>
-      <c r="J64" s="40" t="n"/>
+      <c r="J64" s="40" t="inlineStr"/>
       <c r="K64" s="41" t="n"/>
-      <c r="L64" s="39" t="n"/>
+      <c r="L64" s="39" t="inlineStr"/>
       <c r="M64" s="41" t="n"/>
       <c r="N64" s="42" t="n"/>
-      <c r="O64" s="40" t="n"/>
+      <c r="O64" s="40" t="inlineStr"/>
       <c r="P64" s="39">
         <f>IF(B64="","",IF(L64="Yes","LMS Completed (Ready for Exam)",IF(L64="In Progress","LMS In Progress",IF(H64="Yes","ADD Attended - Awaiting LMS",IF(H64="Rescheduled","ADD Rescheduled",IF(H64="Pending","ADD Scheduled",IF(H64="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q64" s="40" t="n"/>
+      <c r="Q64" s="40" t="inlineStr"/>
       <c r="R64" s="41" t="n"/>
-      <c r="S64" s="40" t="n"/>
+      <c r="S64" s="40" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="35">
         <f>IF(B65="","","REC-"&amp;TEXT(65-8,"000"))</f>
         <v/>
       </c>
-      <c r="B65" s="36" t="n"/>
-      <c r="C65" s="35" t="n"/>
-      <c r="D65" s="36" t="n"/>
-      <c r="E65" s="36" t="n"/>
+      <c r="B65" s="36" t="inlineStr"/>
+      <c r="C65" s="35" t="inlineStr"/>
+      <c r="D65" s="36" t="inlineStr"/>
+      <c r="E65" s="36" t="inlineStr"/>
       <c r="F65" s="37" t="n"/>
       <c r="G65" s="37" t="n"/>
-      <c r="H65" s="35" t="n"/>
+      <c r="H65" s="35" t="inlineStr"/>
       <c r="I65" s="37" t="n"/>
-      <c r="J65" s="36" t="n"/>
+      <c r="J65" s="36" t="inlineStr"/>
       <c r="K65" s="37" t="n"/>
-      <c r="L65" s="35" t="n"/>
+      <c r="L65" s="35" t="inlineStr"/>
       <c r="M65" s="37" t="n"/>
       <c r="N65" s="38" t="n"/>
-      <c r="O65" s="36" t="n"/>
+      <c r="O65" s="36" t="inlineStr"/>
       <c r="P65" s="35">
         <f>IF(B65="","",IF(L65="Yes","LMS Completed (Ready for Exam)",IF(L65="In Progress","LMS In Progress",IF(H65="Yes","ADD Attended - Awaiting LMS",IF(H65="Rescheduled","ADD Rescheduled",IF(H65="Pending","ADD Scheduled",IF(H65="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q65" s="36" t="n"/>
+      <c r="Q65" s="36" t="inlineStr"/>
       <c r="R65" s="37" t="n"/>
-      <c r="S65" s="36" t="n"/>
+      <c r="S65" s="36" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -4001,10 +3259,9 @@
         <f>'Recruit Monitoring Tracker'!B5</f>
         <v/>
       </c>
-      <c r="C6" s="48" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
+      <c r="C6" s="48">
+        <f>IFERROR(B6/B6,1)</f>
+        <v/>
       </c>
       <c r="D6" s="49" t="inlineStr">
         <is>
@@ -5042,7 +4299,7 @@
       </c>
       <c r="B18" s="77" t="inlineStr">
         <is>
-          <t>Rows 24 to 65 are pre-formatted with all dropdowns, formulas, and borders. Simply start typing in Column B (Complete Name), and the entire row will activate automatically!</t>
+          <t>Rows 10 to 65 are pre-formatted with all dropdowns, formulas, and borders. Simply start typing in Column B (Complete Name), and the entire row will activate automatically!</t>
         </is>
       </c>
       <c r="C18" s="78" t="n"/>

</xml_diff>

<commit_message>
Add recruits: Michael Bagiuos, Alona Barilea, Lorenz Garrucha, Princess Ambos, Jezreel Kate Montano
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -1589,139 +1589,294 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="39">
-        <f>IF(B10="","","REC-"&amp;TEXT(10-8,"000"))</f>
-        <v/>
-      </c>
-      <c r="B10" s="40" t="inlineStr"/>
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>REC-002</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Bagiuos, Michael</t>
+        </is>
+      </c>
       <c r="C10" s="39" t="inlineStr"/>
       <c r="D10" s="40" t="inlineStr"/>
       <c r="E10" s="40" t="inlineStr"/>
-      <c r="F10" s="41" t="n"/>
+      <c r="F10" s="41" t="n">
+        <v>46280</v>
+      </c>
       <c r="G10" s="41" t="n"/>
-      <c r="H10" s="39" t="inlineStr"/>
+      <c r="H10" s="39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I10" s="41" t="n"/>
-      <c r="J10" s="40" t="inlineStr"/>
+      <c r="J10" s="40" t="inlineStr">
+        <is>
+          <t>Newly added recruit; pending ADD orientation schedule.</t>
+        </is>
+      </c>
       <c r="K10" s="41" t="n"/>
-      <c r="L10" s="39" t="inlineStr"/>
+      <c r="L10" s="39" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="M10" s="41" t="n"/>
-      <c r="N10" s="42" t="n"/>
+      <c r="N10" s="42" t="n">
+        <v>0</v>
+      </c>
       <c r="O10" s="40" t="inlineStr"/>
       <c r="P10" s="39">
         <f>IF(B10="","",IF(L10="Yes","LMS Completed (Ready for Exam)",IF(L10="In Progress","LMS In Progress",IF(H10="Yes","ADD Attended - Awaiting LMS",IF(H10="Rescheduled","ADD Rescheduled",IF(H10="Pending","ADD Scheduled",IF(H10="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q10" s="40" t="inlineStr"/>
-      <c r="R10" s="41" t="n"/>
-      <c r="S10" s="40" t="inlineStr"/>
+      <c r="Q10" s="40" t="inlineStr">
+        <is>
+          <t>Confirm ADD schedule &amp; send orientation invite</t>
+        </is>
+      </c>
+      <c r="R10" s="41" t="n">
+        <v>46281</v>
+      </c>
+      <c r="S10" s="40" t="inlineStr">
+        <is>
+          <t>Recruit added to monitoring pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="35">
-        <f>IF(B11="","","REC-"&amp;TEXT(11-8,"000"))</f>
-        <v/>
-      </c>
-      <c r="B11" s="36" t="inlineStr"/>
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>REC-003</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>Barilea, Alona</t>
+        </is>
+      </c>
       <c r="C11" s="35" t="inlineStr"/>
       <c r="D11" s="36" t="inlineStr"/>
       <c r="E11" s="36" t="inlineStr"/>
-      <c r="F11" s="37" t="n"/>
+      <c r="F11" s="37" t="n">
+        <v>46280</v>
+      </c>
       <c r="G11" s="37" t="n"/>
-      <c r="H11" s="35" t="inlineStr"/>
+      <c r="H11" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I11" s="37" t="n"/>
-      <c r="J11" s="36" t="inlineStr"/>
+      <c r="J11" s="36" t="inlineStr">
+        <is>
+          <t>Newly added recruit; pending ADD orientation schedule.</t>
+        </is>
+      </c>
       <c r="K11" s="37" t="n"/>
-      <c r="L11" s="35" t="inlineStr"/>
+      <c r="L11" s="35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="M11" s="37" t="n"/>
-      <c r="N11" s="38" t="n"/>
+      <c r="N11" s="38" t="n">
+        <v>0</v>
+      </c>
       <c r="O11" s="36" t="inlineStr"/>
       <c r="P11" s="35">
         <f>IF(B11="","",IF(L11="Yes","LMS Completed (Ready for Exam)",IF(L11="In Progress","LMS In Progress",IF(H11="Yes","ADD Attended - Awaiting LMS",IF(H11="Rescheduled","ADD Rescheduled",IF(H11="Pending","ADD Scheduled",IF(H11="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q11" s="36" t="inlineStr"/>
-      <c r="R11" s="37" t="n"/>
-      <c r="S11" s="36" t="inlineStr"/>
+      <c r="Q11" s="36" t="inlineStr">
+        <is>
+          <t>Confirm ADD schedule &amp; send orientation invite</t>
+        </is>
+      </c>
+      <c r="R11" s="37" t="n">
+        <v>46281</v>
+      </c>
+      <c r="S11" s="36" t="inlineStr">
+        <is>
+          <t>Recruit added to monitoring pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="39">
-        <f>IF(B12="","","REC-"&amp;TEXT(12-8,"000"))</f>
-        <v/>
-      </c>
-      <c r="B12" s="40" t="inlineStr"/>
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>REC-004</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Garrucha, Lorenz</t>
+        </is>
+      </c>
       <c r="C12" s="39" t="inlineStr"/>
       <c r="D12" s="40" t="inlineStr"/>
       <c r="E12" s="40" t="inlineStr"/>
-      <c r="F12" s="41" t="n"/>
+      <c r="F12" s="41" t="n">
+        <v>46280</v>
+      </c>
       <c r="G12" s="41" t="n"/>
-      <c r="H12" s="39" t="inlineStr"/>
+      <c r="H12" s="39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I12" s="41" t="n"/>
-      <c r="J12" s="40" t="inlineStr"/>
+      <c r="J12" s="40" t="inlineStr">
+        <is>
+          <t>Newly added recruit; pending ADD orientation schedule.</t>
+        </is>
+      </c>
       <c r="K12" s="41" t="n"/>
-      <c r="L12" s="39" t="inlineStr"/>
+      <c r="L12" s="39" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="M12" s="41" t="n"/>
-      <c r="N12" s="42" t="n"/>
+      <c r="N12" s="42" t="n">
+        <v>0</v>
+      </c>
       <c r="O12" s="40" t="inlineStr"/>
       <c r="P12" s="39">
         <f>IF(B12="","",IF(L12="Yes","LMS Completed (Ready for Exam)",IF(L12="In Progress","LMS In Progress",IF(H12="Yes","ADD Attended - Awaiting LMS",IF(H12="Rescheduled","ADD Rescheduled",IF(H12="Pending","ADD Scheduled",IF(H12="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q12" s="40" t="inlineStr"/>
-      <c r="R12" s="41" t="n"/>
-      <c r="S12" s="40" t="inlineStr"/>
+      <c r="Q12" s="40" t="inlineStr">
+        <is>
+          <t>Confirm ADD schedule &amp; send orientation invite</t>
+        </is>
+      </c>
+      <c r="R12" s="41" t="n">
+        <v>46281</v>
+      </c>
+      <c r="S12" s="40" t="inlineStr">
+        <is>
+          <t>Recruit added to monitoring pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="35">
-        <f>IF(B13="","","REC-"&amp;TEXT(13-8,"000"))</f>
-        <v/>
-      </c>
-      <c r="B13" s="36" t="inlineStr"/>
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>REC-005</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>Ambos, Princess</t>
+        </is>
+      </c>
       <c r="C13" s="35" t="inlineStr"/>
       <c r="D13" s="36" t="inlineStr"/>
       <c r="E13" s="36" t="inlineStr"/>
-      <c r="F13" s="37" t="n"/>
+      <c r="F13" s="37" t="n">
+        <v>46280</v>
+      </c>
       <c r="G13" s="37" t="n"/>
-      <c r="H13" s="35" t="inlineStr"/>
+      <c r="H13" s="35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I13" s="37" t="n"/>
-      <c r="J13" s="36" t="inlineStr"/>
+      <c r="J13" s="36" t="inlineStr">
+        <is>
+          <t>Newly added recruit; pending ADD orientation schedule.</t>
+        </is>
+      </c>
       <c r="K13" s="37" t="n"/>
-      <c r="L13" s="35" t="inlineStr"/>
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="M13" s="37" t="n"/>
-      <c r="N13" s="38" t="n"/>
+      <c r="N13" s="38" t="n">
+        <v>0</v>
+      </c>
       <c r="O13" s="36" t="inlineStr"/>
       <c r="P13" s="35">
         <f>IF(B13="","",IF(L13="Yes","LMS Completed (Ready for Exam)",IF(L13="In Progress","LMS In Progress",IF(H13="Yes","ADD Attended - Awaiting LMS",IF(H13="Rescheduled","ADD Rescheduled",IF(H13="Pending","ADD Scheduled",IF(H13="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q13" s="36" t="inlineStr"/>
-      <c r="R13" s="37" t="n"/>
-      <c r="S13" s="36" t="inlineStr"/>
+      <c r="Q13" s="36" t="inlineStr">
+        <is>
+          <t>Confirm ADD schedule &amp; send orientation invite</t>
+        </is>
+      </c>
+      <c r="R13" s="37" t="n">
+        <v>46281</v>
+      </c>
+      <c r="S13" s="36" t="inlineStr">
+        <is>
+          <t>Recruit added to monitoring pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="39">
-        <f>IF(B14="","","REC-"&amp;TEXT(14-8,"000"))</f>
-        <v/>
-      </c>
-      <c r="B14" s="40" t="inlineStr"/>
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>REC-006</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>Montano, Jezreel Kate</t>
+        </is>
+      </c>
       <c r="C14" s="39" t="inlineStr"/>
       <c r="D14" s="40" t="inlineStr"/>
       <c r="E14" s="40" t="inlineStr"/>
-      <c r="F14" s="41" t="n"/>
+      <c r="F14" s="41" t="n">
+        <v>46280</v>
+      </c>
       <c r="G14" s="41" t="n"/>
-      <c r="H14" s="39" t="inlineStr"/>
+      <c r="H14" s="39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I14" s="41" t="n"/>
-      <c r="J14" s="40" t="inlineStr"/>
+      <c r="J14" s="40" t="inlineStr">
+        <is>
+          <t>Newly added recruit; pending ADD orientation schedule.</t>
+        </is>
+      </c>
       <c r="K14" s="41" t="n"/>
-      <c r="L14" s="39" t="inlineStr"/>
+      <c r="L14" s="39" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="M14" s="41" t="n"/>
-      <c r="N14" s="42" t="n"/>
+      <c r="N14" s="42" t="n">
+        <v>0</v>
+      </c>
       <c r="O14" s="40" t="inlineStr"/>
       <c r="P14" s="39">
         <f>IF(B14="","",IF(L14="Yes","LMS Completed (Ready for Exam)",IF(L14="In Progress","LMS In Progress",IF(H14="Yes","ADD Attended - Awaiting LMS",IF(H14="Rescheduled","ADD Rescheduled",IF(H14="Pending","ADD Scheduled",IF(H14="No","ADD Missed - Follow Up","Initial Prospect")))))))</f>
         <v/>
       </c>
-      <c r="Q14" s="40" t="inlineStr"/>
-      <c r="R14" s="41" t="n"/>
-      <c r="S14" s="40" t="inlineStr"/>
+      <c r="Q14" s="40" t="inlineStr">
+        <is>
+          <t>Confirm ADD schedule &amp; send orientation invite</t>
+        </is>
+      </c>
+      <c r="R14" s="41" t="n">
+        <v>46281</v>
+      </c>
+      <c r="S14" s="40" t="inlineStr">
+        <is>
+          <t>Recruit added to monitoring pipeline.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="35">
@@ -4299,7 +4454,7 @@
       </c>
       <c r="B18" s="77" t="inlineStr">
         <is>
-          <t>Rows 10 to 65 are pre-formatted with all dropdowns, formulas, and borders. Simply start typing in Column B (Complete Name), and the entire row will activate automatically!</t>
+          <t>Rows 15 to 65 are pre-formatted with all dropdowns, formulas, and borders. Simply start typing in Column B (Complete Name), and the entire row will activate automatically!</t>
         </is>
       </c>
       <c r="C18" s="78" t="n"/>

</xml_diff>

<commit_message>
Update: All 6 recruits attended ADD Sept 14; Maybe Grandes processing LMS
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -1368,7 +1368,7 @@
       <c r="H6" s="6" t="n"/>
       <c r="J6" s="20" t="inlineStr">
         <is>
-          <t>Currently taking online modules</t>
+          <t>Currently processing modules</t>
         </is>
       </c>
       <c r="K6" s="8" t="n"/>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="J9" s="36" t="inlineStr">
         <is>
-          <t>Attended ADD on Sept 14; confirmed interest. Preparing for LMS setup.</t>
+          <t>Attended ADD on Sept 14; confirmed proceeding with LMS training.</t>
         </is>
       </c>
       <c r="K9" s="37" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="L9" s="35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M9" s="37" t="n"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="O9" s="36" t="inlineStr">
         <is>
-          <t>Pending account activation</t>
+          <t>Account registration in progress</t>
         </is>
       </c>
       <c r="P9" s="35">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="Q9" s="36" t="inlineStr">
         <is>
-          <t>Set up LMS account &amp; send module access link today</t>
+          <t>Process LMS portal registration &amp; send login access link today</t>
         </is>
       </c>
       <c r="R9" s="37" t="n">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="S9" s="36" t="inlineStr">
         <is>
-          <t>Attended ADD yesterday Sept 14, 2026. Will set up her LMS today.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Processing her LMS onboarding today.</t>
         </is>
       </c>
     </row>
@@ -1603,18 +1603,22 @@
       <c r="D10" s="40" t="inlineStr"/>
       <c r="E10" s="40" t="inlineStr"/>
       <c r="F10" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G10" s="41" t="n"/>
+        <v>46279</v>
+      </c>
+      <c r="G10" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="H10" s="39" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I10" s="41" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="J10" s="40" t="inlineStr">
         <is>
-          <t>Newly added recruit; pending ADD orientation schedule.</t>
+          <t>Attended ADD on Sept 14; not yet processing LMS.</t>
         </is>
       </c>
       <c r="K10" s="41" t="n"/>
@@ -1634,7 +1638,7 @@
       </c>
       <c r="Q10" s="40" t="inlineStr">
         <is>
-          <t>Confirm ADD schedule &amp; send orientation invite</t>
+          <t>Follow up on ADD feedback &amp; check readiness to process LMS</t>
         </is>
       </c>
       <c r="R10" s="41" t="n">
@@ -1642,7 +1646,7 @@
       </c>
       <c r="S10" s="40" t="inlineStr">
         <is>
-          <t>Recruit added to monitoring pipeline.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Pending decision to proceed with LMS.</t>
         </is>
       </c>
     </row>
@@ -1661,18 +1665,22 @@
       <c r="D11" s="36" t="inlineStr"/>
       <c r="E11" s="36" t="inlineStr"/>
       <c r="F11" s="37" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G11" s="37" t="n"/>
+        <v>46279</v>
+      </c>
+      <c r="G11" s="37" t="n">
+        <v>46279</v>
+      </c>
       <c r="H11" s="35" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I11" s="37" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I11" s="37" t="n">
+        <v>46279</v>
+      </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Newly added recruit; pending ADD orientation schedule.</t>
+          <t>Attended ADD on Sept 14; not yet processing LMS.</t>
         </is>
       </c>
       <c r="K11" s="37" t="n"/>
@@ -1692,7 +1700,7 @@
       </c>
       <c r="Q11" s="36" t="inlineStr">
         <is>
-          <t>Confirm ADD schedule &amp; send orientation invite</t>
+          <t>Follow up on ADD feedback &amp; check readiness to process LMS</t>
         </is>
       </c>
       <c r="R11" s="37" t="n">
@@ -1700,7 +1708,7 @@
       </c>
       <c r="S11" s="36" t="inlineStr">
         <is>
-          <t>Recruit added to monitoring pipeline.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Pending decision to proceed with LMS.</t>
         </is>
       </c>
     </row>
@@ -1719,18 +1727,22 @@
       <c r="D12" s="40" t="inlineStr"/>
       <c r="E12" s="40" t="inlineStr"/>
       <c r="F12" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G12" s="41" t="n"/>
+        <v>46279</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="H12" s="39" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I12" s="41" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I12" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="J12" s="40" t="inlineStr">
         <is>
-          <t>Newly added recruit; pending ADD orientation schedule.</t>
+          <t>Attended ADD on Sept 14; not yet processing LMS.</t>
         </is>
       </c>
       <c r="K12" s="41" t="n"/>
@@ -1750,7 +1762,7 @@
       </c>
       <c r="Q12" s="40" t="inlineStr">
         <is>
-          <t>Confirm ADD schedule &amp; send orientation invite</t>
+          <t>Follow up on ADD feedback &amp; check readiness to process LMS</t>
         </is>
       </c>
       <c r="R12" s="41" t="n">
@@ -1758,7 +1770,7 @@
       </c>
       <c r="S12" s="40" t="inlineStr">
         <is>
-          <t>Recruit added to monitoring pipeline.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Pending decision to proceed with LMS.</t>
         </is>
       </c>
     </row>
@@ -1777,18 +1789,22 @@
       <c r="D13" s="36" t="inlineStr"/>
       <c r="E13" s="36" t="inlineStr"/>
       <c r="F13" s="37" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G13" s="37" t="n"/>
+        <v>46279</v>
+      </c>
+      <c r="G13" s="37" t="n">
+        <v>46279</v>
+      </c>
       <c r="H13" s="35" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I13" s="37" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I13" s="37" t="n">
+        <v>46279</v>
+      </c>
       <c r="J13" s="36" t="inlineStr">
         <is>
-          <t>Newly added recruit; pending ADD orientation schedule.</t>
+          <t>Attended ADD on Sept 14; not yet processing LMS.</t>
         </is>
       </c>
       <c r="K13" s="37" t="n"/>
@@ -1808,7 +1824,7 @@
       </c>
       <c r="Q13" s="36" t="inlineStr">
         <is>
-          <t>Confirm ADD schedule &amp; send orientation invite</t>
+          <t>Follow up on ADD feedback &amp; check readiness to process LMS</t>
         </is>
       </c>
       <c r="R13" s="37" t="n">
@@ -1816,7 +1832,7 @@
       </c>
       <c r="S13" s="36" t="inlineStr">
         <is>
-          <t>Recruit added to monitoring pipeline.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Pending decision to proceed with LMS.</t>
         </is>
       </c>
     </row>
@@ -1835,18 +1851,22 @@
       <c r="D14" s="40" t="inlineStr"/>
       <c r="E14" s="40" t="inlineStr"/>
       <c r="F14" s="41" t="n">
-        <v>46280</v>
-      </c>
-      <c r="G14" s="41" t="n"/>
+        <v>46279</v>
+      </c>
+      <c r="G14" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="H14" s="39" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I14" s="41" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I14" s="41" t="n">
+        <v>46279</v>
+      </c>
       <c r="J14" s="40" t="inlineStr">
         <is>
-          <t>Newly added recruit; pending ADD orientation schedule.</t>
+          <t>Attended ADD on Sept 14; not yet processing LMS.</t>
         </is>
       </c>
       <c r="K14" s="41" t="n"/>
@@ -1866,7 +1886,7 @@
       </c>
       <c r="Q14" s="40" t="inlineStr">
         <is>
-          <t>Confirm ADD schedule &amp; send orientation invite</t>
+          <t>Follow up on ADD feedback &amp; check readiness to process LMS</t>
         </is>
       </c>
       <c r="R14" s="41" t="n">
@@ -1874,7 +1894,7 @@
       </c>
       <c r="S14" s="40" t="inlineStr">
         <is>
-          <t>Recruit added to monitoring pipeline.</t>
+          <t>Attended ADD yesterday Sept 14, 2026. Pending decision to proceed with LMS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add downloadable ADD Registration Form (.html) and embedded Excel registration slip tab
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Recruitment Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Dropdowns &amp; Settings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="User Guide &amp; Workflow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ADD Registration Form" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -145,8 +146,43 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00E2E8F0"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -255,8 +291,14 @@
         <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -376,11 +418,60 @@
         <color rgb="001E3A8A"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -580,6 +671,23 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4583,4 +4691,406 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="79" t="inlineStr">
+        <is>
+          <t>AGENCY DISCOVERY DAY (ADD) — REGISTRATION FORM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>Candidate Career Orientation Intake Slip | Pre-Licensing Recruitment Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="75" t="inlineStr">
+        <is>
+          <t>1. CANDIDATE PERSONAL INFORMATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="81" t="inlineStr">
+        <is>
+          <t>Complete Name:</t>
+        </is>
+      </c>
+      <c r="B5" s="82" t="inlineStr">
+        <is>
+          <t>Last Name, First Name M.I.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="81" t="inlineStr">
+        <is>
+          <t>Mobile Number:</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>+63 9XX XXX XXXX</t>
+        </is>
+      </c>
+      <c r="D6" s="81" t="inlineStr">
+        <is>
+          <t>Email Address:</t>
+        </is>
+      </c>
+      <c r="E6" s="82" t="inlineStr">
+        <is>
+          <t>candidate@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="81" t="inlineStr">
+        <is>
+          <t>Date of Birth:</t>
+        </is>
+      </c>
+      <c r="B7" s="82" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="D7" s="81" t="inlineStr">
+        <is>
+          <t>Civil Status:</t>
+        </is>
+      </c>
+      <c r="E7" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Single   [ ] Married   [ ] Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="81" t="inlineStr">
+        <is>
+          <t>City / Address:</t>
+        </is>
+      </c>
+      <c r="B8" s="82" t="inlineStr">
+        <is>
+          <t>City, Province</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="6" customHeight="1"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="75" t="inlineStr">
+        <is>
+          <t>2. BACKGROUND &amp; CURRENT OCCUPATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="81" t="inlineStr">
+        <is>
+          <t>Current Field:</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Employed   [ ] Business   [ ] Freelance</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>Current Company / Role:</t>
+        </is>
+      </c>
+      <c r="E11" s="82" t="inlineStr">
+        <is>
+          <t>Job Title / Employer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>Education:</t>
+        </is>
+      </c>
+      <c r="B12" s="82" t="inlineStr">
+        <is>
+          <t>College Degree / Course</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>Work Experience:</t>
+        </is>
+      </c>
+      <c r="E12" s="83" t="inlineStr">
+        <is>
+          <t>[ ] &lt;1 yr   [ ] 1-3 yrs   [ ] 3-5 yrs   [ ] 5+ yrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="6" customHeight="1"/>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="75" t="inlineStr">
+        <is>
+          <t>3. SOURCING &amp; ADD ORIENTATION SCHEDULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="81" t="inlineStr">
+        <is>
+          <t>Invited By (Recruiter):</t>
+        </is>
+      </c>
+      <c r="B15" s="82" t="inlineStr">
+        <is>
+          <t>Recruiter / Unit Manager Name</t>
+        </is>
+      </c>
+      <c r="D15" s="81" t="inlineStr">
+        <is>
+          <t>Date Invited / Sourced:</t>
+        </is>
+      </c>
+      <c r="E15" s="83" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="81" t="inlineStr">
+        <is>
+          <t>Preferred ADD Session:</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Saturday Morning (10 AM)   [ ] Saturday Afternoon (2 PM)</t>
+        </is>
+      </c>
+      <c r="D16" s="81" t="inlineStr">
+        <is>
+          <t>Orientation Mode:</t>
+        </is>
+      </c>
+      <c r="E16" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Online via Zoom   [ ] Branch / In-Person</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="6" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="75" t="inlineStr">
+        <is>
+          <t>4. MOTIVATION &amp; CAREER OBJECTIVES</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="81" t="inlineStr">
+        <is>
+          <t>Primary Motivation:</t>
+        </is>
+      </c>
+      <c r="B19" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Unlimited Income Potential   [ ] Flexible Time   [ ] Work from Home   [ ] Helping Others</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="81" t="inlineStr">
+        <is>
+          <t>Career Mode:</t>
+        </is>
+      </c>
+      <c r="B20" s="83" t="inlineStr">
+        <is>
+          <t>[ ] Full-Time Financial Advisor     [ ] Part-Time Financial Advisor     [ ] Exploring / Open-Minded</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="75" t="inlineStr">
+        <is>
+          <t>5. CONFIRMATION &amp; OFFICE USE ONLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="81" t="inlineStr">
+        <is>
+          <t>Candidate Signature:</t>
+        </is>
+      </c>
+      <c r="B23" s="84" t="inlineStr">
+        <is>
+          <t>____________________________</t>
+        </is>
+      </c>
+      <c r="D23" s="81" t="inlineStr">
+        <is>
+          <t>Date Signed:</t>
+        </is>
+      </c>
+      <c r="E23" s="84" t="inlineStr">
+        <is>
+          <t>____________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="85" t="inlineStr">
+        <is>
+          <t>--- FOR AGENCY / UNIT MANAGER USE ONLY ---</t>
+        </is>
+      </c>
+      <c r="B24" s="86" t="n"/>
+      <c r="C24" s="86" t="n"/>
+      <c r="D24" s="86" t="n"/>
+      <c r="E24" s="86" t="n"/>
+      <c r="F24" s="86" t="n"/>
+      <c r="G24" s="87" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="88" t="inlineStr">
+        <is>
+          <t>Assigned Recruit ID:</t>
+        </is>
+      </c>
+      <c r="B25" s="89" t="inlineStr">
+        <is>
+          <t>REC-_____</t>
+        </is>
+      </c>
+      <c r="C25" s="87" t="n"/>
+      <c r="D25" s="88" t="inlineStr">
+        <is>
+          <t>ADD Attendance:</t>
+        </is>
+      </c>
+      <c r="E25" s="89" t="inlineStr">
+        <is>
+          <t>[ ] Attended (Date: ________)   [ ] Rescheduled</t>
+        </is>
+      </c>
+      <c r="F25" s="86" t="n"/>
+      <c r="G25" s="87" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="88" t="inlineStr">
+        <is>
+          <t>LMS Endorsement:</t>
+        </is>
+      </c>
+      <c r="B26" s="89" t="inlineStr">
+        <is>
+          <t>[ ] Approved for LMS Modules</t>
+        </is>
+      </c>
+      <c r="C26" s="87" t="n"/>
+      <c r="D26" s="88" t="inlineStr">
+        <is>
+          <t>LMS Setup Date:</t>
+        </is>
+      </c>
+      <c r="E26" s="89" t="inlineStr">
+        <is>
+          <t>Credentials Sent Date: ________</t>
+        </is>
+      </c>
+      <c r="F26" s="86" t="n"/>
+      <c r="G26" s="87" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="88" t="inlineStr">
+        <is>
+          <t>UM / Recruiter Sign:</t>
+        </is>
+      </c>
+      <c r="B27" s="89" t="inlineStr">
+        <is>
+          <t>_______________________</t>
+        </is>
+      </c>
+      <c r="C27" s="87" t="n"/>
+      <c r="D27" s="88" t="inlineStr">
+        <is>
+          <t>Overall Status:</t>
+        </is>
+      </c>
+      <c r="E27" s="89" t="inlineStr">
+        <is>
+          <t>[ ] Active In Pipeline   [ ] Ready for Exam</t>
+        </is>
+      </c>
+      <c r="F27" s="86" t="n"/>
+      <c r="G27" s="87" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="32">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B26:C26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update next ADD date to Thursday, September 17, 2026 across tracker, form, and emails
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -3887,15 +3887,15 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="46" t="inlineStr">
         <is>
-          <t>Sarah Jenkins (UM)</t>
+          <t>Cedric (cedric.axa1@gmail.com)</t>
         </is>
       </c>
       <c r="B22" s="47">
-        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*")</f>
+        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Cedric (cedric.axa1@gmail.com)*")</f>
         <v/>
       </c>
       <c r="C22" s="65">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Cedric (cedric.axa1@gmail.com)*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
         <v/>
       </c>
       <c r="D22" s="38">
@@ -3903,7 +3903,7 @@
         <v/>
       </c>
       <c r="E22" s="65">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Cedric (cedric.axa1@gmail.com)*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
         <v/>
       </c>
       <c r="F22" s="38">
@@ -3911,22 +3911,22 @@
         <v/>
       </c>
       <c r="G22" s="47">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Cedric (cedric.axa1@gmail.com)*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="50" t="inlineStr">
         <is>
-          <t>David Tan</t>
+          <t>Sarah Jenkins (UM)</t>
         </is>
       </c>
       <c r="B23" s="51">
-        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*David Tan*")</f>
+        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*")</f>
         <v/>
       </c>
       <c r="C23" s="66">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
         <v/>
       </c>
       <c r="D23" s="42">
@@ -3934,7 +3934,7 @@
         <v/>
       </c>
       <c r="E23" s="66">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
         <v/>
       </c>
       <c r="F23" s="42">
@@ -3942,22 +3942,22 @@
         <v/>
       </c>
       <c r="G23" s="51">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="46" t="inlineStr">
         <is>
-          <t>Elena Gomez</t>
+          <t>David Tan</t>
         </is>
       </c>
       <c r="B24" s="47">
-        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*")</f>
+        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*David Tan*")</f>
         <v/>
       </c>
       <c r="C24" s="65">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
         <v/>
       </c>
       <c r="D24" s="38">
@@ -3965,7 +3965,7 @@
         <v/>
       </c>
       <c r="E24" s="65">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
         <v/>
       </c>
       <c r="F24" s="38">
@@ -3973,22 +3973,22 @@
         <v/>
       </c>
       <c r="G24" s="47">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*David Tan*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="50" t="inlineStr">
         <is>
-          <t>Michael Chang</t>
+          <t>Elena Gomez</t>
         </is>
       </c>
       <c r="B25" s="51">
-        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Michael Chang*")</f>
+        <f>COUNTIF('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*")</f>
         <v/>
       </c>
       <c r="C25" s="66">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Michael Chang*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!H9:H65, "Yes")</f>
         <v/>
       </c>
       <c r="D25" s="42">
@@ -3996,7 +3996,7 @@
         <v/>
       </c>
       <c r="E25" s="66">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Michael Chang*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!L9:L65, "Yes")</f>
         <v/>
       </c>
       <c r="F25" s="42">
@@ -4004,7 +4004,7 @@
         <v/>
       </c>
       <c r="G25" s="51">
-        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Michael Chang*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
+        <f>COUNTIFS('Recruit Monitoring Tracker'!E9:E65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!P9:P65, "*Ready for Exam*")</f>
         <v/>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="B16" s="83" t="inlineStr">
         <is>
-          <t>[ ] Saturday Morning (10 AM)   [ ] Saturday Afternoon (2 PM)</t>
+          <t>[X] Thursday, Sept 17, 2026 (Next ADD)   [ ] Special / Alternate Date</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">

</xml_diff>

<commit_message>
Restrict all ADD session options exclusively to Thursdays at 7:00 PM
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -4922,12 +4922,12 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="81" t="inlineStr">
         <is>
-          <t>Preferred ADD Session:</t>
+          <t>ADD Session (Thursdays 7 PM):</t>
         </is>
       </c>
       <c r="B16" s="83" t="inlineStr">
         <is>
-          <t>[X] Thursday, Sept 17, 2026 (7:00 PM)   [ ] Special / Alternate Date</t>
+          <t>[X] Thursday, Sept 17 (7 PM)   [ ] Thursday, Sept 24 (7 PM)   [ ] Future Thursday</t>
         </is>
       </c>
       <c r="D16" s="81" t="inlineStr">

</xml_diff>

<commit_message>
Add Sheet 6 Recruiter Directory & IDs and web upload portal for Recruiter IDs
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Recruit_Monitoring_Tracker.xlsx
+++ b/Recruit_Monitoring_Tracker.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Dropdowns &amp; Settings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="User Guide &amp; Workflow" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ADD Registration Form" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Recruiter Directory &amp; IDs" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -179,6 +180,48 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
       <sz val="9.5"/>
     </font>
   </fonts>
@@ -471,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -688,6 +731,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="19" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="19" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="29" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="31" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="33" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5129,4 +5229,1329 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AGENCY RECRUITER DIRECTORY &amp; IDENTIFICATION ROSTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="90" t="inlineStr">
+        <is>
+          <t>Official Recruiter IDs, Agent Codes, Contact Details, License Credentials &amp; Performance Metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="16" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL RECRUITERS</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE STATUS</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL SOURCED</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="8" t="n"/>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>ADD ATTENDED</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="n"/>
+      <c r="M4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="B5" s="91">
+        <f>COUNTA(A9:A35)</f>
+        <v/>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="92">
+        <f>COUNTIF(H9:H35, "Active")</f>
+        <v/>
+      </c>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="93">
+        <f>SUM(J9:J35)</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="94">
+        <f>SUM(K9:K35)</f>
+        <v/>
+      </c>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Authorized agency recruiters</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Currently sourcing talent</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Total candidates invited</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8" t="n"/>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>Candidates attended ADD</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="8" customHeight="1"/>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="95" t="inlineStr">
+        <is>
+          <t>Recruiter ID / Code</t>
+        </is>
+      </c>
+      <c r="B8" s="96" t="inlineStr">
+        <is>
+          <t>Recruiter Full Name</t>
+        </is>
+      </c>
+      <c r="C8" s="96" t="inlineStr">
+        <is>
+          <t>Email Address</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="inlineStr">
+        <is>
+          <t>Contact Number</t>
+        </is>
+      </c>
+      <c r="E8" s="96" t="inlineStr">
+        <is>
+          <t>Agency Unit / Team</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>License / IC Code</t>
+        </is>
+      </c>
+      <c r="G8" s="96" t="inlineStr">
+        <is>
+          <t>Gov ID / Verification</t>
+        </is>
+      </c>
+      <c r="H8" s="95" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="95" t="inlineStr">
+        <is>
+          <t>Date Added</t>
+        </is>
+      </c>
+      <c r="J8" s="95" t="inlineStr">
+        <is>
+          <t>Recruits Sourced</t>
+        </is>
+      </c>
+      <c r="K8" s="95" t="inlineStr">
+        <is>
+          <t>Attended ADD</t>
+        </is>
+      </c>
+      <c r="L8" s="95" t="inlineStr">
+        <is>
+          <t>LMS In Progress</t>
+        </is>
+      </c>
+      <c r="M8" s="95" t="inlineStr">
+        <is>
+          <t>LMS Completed</t>
+        </is>
+      </c>
+      <c r="N8" s="96" t="inlineStr">
+        <is>
+          <t>ID File Reference / Upload Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="97" t="inlineStr">
+        <is>
+          <t>AGT-001</t>
+        </is>
+      </c>
+      <c r="B9" s="98" t="inlineStr">
+        <is>
+          <t>Cedric</t>
+        </is>
+      </c>
+      <c r="C9" s="99" t="inlineStr">
+        <is>
+          <t>cedric.axa1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D9" s="100" t="inlineStr">
+        <is>
+          <t>0917 888 9999</t>
+        </is>
+      </c>
+      <c r="E9" s="99" t="inlineStr">
+        <is>
+          <t>Executive Agency Unit</t>
+        </is>
+      </c>
+      <c r="F9" s="100" t="inlineStr">
+        <is>
+          <t>LIC-2024-001</t>
+        </is>
+      </c>
+      <c r="G9" s="99" t="inlineStr">
+        <is>
+          <t>PRC Professional License</t>
+        </is>
+      </c>
+      <c r="H9" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I9" s="100" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="J9" s="101">
+        <f>COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*Cedric*")</f>
+        <v/>
+      </c>
+      <c r="K9" s="101">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Cedric*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="L9" s="102">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Cedric*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress")</f>
+        <v/>
+      </c>
+      <c r="M9" s="102">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Cedric*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="N9" s="99" t="inlineStr">
+        <is>
+          <t>Verified / Primary Recruiter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="103" t="inlineStr">
+        <is>
+          <t>AGT-002</t>
+        </is>
+      </c>
+      <c r="B10" s="104" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins (UM)</t>
+        </is>
+      </c>
+      <c r="C10" s="105" t="inlineStr">
+        <is>
+          <t>sarah.jenkins@agency.com</t>
+        </is>
+      </c>
+      <c r="D10" s="106" t="inlineStr">
+        <is>
+          <t>0918 222 3333</t>
+        </is>
+      </c>
+      <c r="E10" s="105" t="inlineStr">
+        <is>
+          <t>Alpha Leaders Unit</t>
+        </is>
+      </c>
+      <c r="F10" s="106" t="inlineStr">
+        <is>
+          <t>LIC-2023-088</t>
+        </is>
+      </c>
+      <c r="G10" s="105" t="inlineStr">
+        <is>
+          <t>Unified Multi-Purpose ID</t>
+        </is>
+      </c>
+      <c r="H10" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I10" s="106" t="inlineStr">
+        <is>
+          <t>2023-06-01</t>
+        </is>
+      </c>
+      <c r="J10" s="107">
+        <f>COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*Sarah Jenkins (UM)*")</f>
+        <v/>
+      </c>
+      <c r="K10" s="107">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="L10" s="108">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress")</f>
+        <v/>
+      </c>
+      <c r="M10" s="108">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Sarah Jenkins (UM)*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="N10" s="105" t="inlineStr">
+        <is>
+          <t>Verified / Unit Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="97" t="inlineStr">
+        <is>
+          <t>AGT-003</t>
+        </is>
+      </c>
+      <c r="B11" s="98" t="inlineStr">
+        <is>
+          <t>David Tan</t>
+        </is>
+      </c>
+      <c r="C11" s="99" t="inlineStr">
+        <is>
+          <t>david.tan@agency.com</t>
+        </is>
+      </c>
+      <c r="D11" s="100" t="inlineStr">
+        <is>
+          <t>0919 444 5555</t>
+        </is>
+      </c>
+      <c r="E11" s="99" t="inlineStr">
+        <is>
+          <t>Apex Financial Team</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
+          <t>LIC-2024-112</t>
+        </is>
+      </c>
+      <c r="G11" s="99" t="inlineStr">
+        <is>
+          <t>Passport / Driver's License</t>
+        </is>
+      </c>
+      <c r="H11" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I11" s="100" t="inlineStr">
+        <is>
+          <t>2024-02-10</t>
+        </is>
+      </c>
+      <c r="J11" s="101">
+        <f>COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*David Tan*")</f>
+        <v/>
+      </c>
+      <c r="K11" s="101">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*David Tan*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="L11" s="102">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*David Tan*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress")</f>
+        <v/>
+      </c>
+      <c r="M11" s="102">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*David Tan*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="N11" s="99" t="inlineStr">
+        <is>
+          <t>Verified / Agency Leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="103" t="inlineStr">
+        <is>
+          <t>AGT-004</t>
+        </is>
+      </c>
+      <c r="B12" s="104" t="inlineStr">
+        <is>
+          <t>Elena Gomez</t>
+        </is>
+      </c>
+      <c r="C12" s="105" t="inlineStr">
+        <is>
+          <t>elena.gomez@agency.com</t>
+        </is>
+      </c>
+      <c r="D12" s="106" t="inlineStr">
+        <is>
+          <t>0920 666 7777</t>
+        </is>
+      </c>
+      <c r="E12" s="105" t="inlineStr">
+        <is>
+          <t>Summit Advisors Unit</t>
+        </is>
+      </c>
+      <c r="F12" s="106" t="inlineStr">
+        <is>
+          <t>LIC-2024-190</t>
+        </is>
+      </c>
+      <c r="G12" s="105" t="inlineStr">
+        <is>
+          <t>PRC License ID</t>
+        </is>
+      </c>
+      <c r="H12" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I12" s="106" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="J12" s="107">
+        <f>COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*Elena Gomez*")</f>
+        <v/>
+      </c>
+      <c r="K12" s="107">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="L12" s="108">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress")</f>
+        <v/>
+      </c>
+      <c r="M12" s="108">
+        <f>COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*Elena Gomez*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes")</f>
+        <v/>
+      </c>
+      <c r="N12" s="105" t="inlineStr">
+        <is>
+          <t>Verified / Unit Leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="97" t="inlineStr">
+        <is>
+          <t>AGT-005</t>
+        </is>
+      </c>
+      <c r="B13" s="98" t="inlineStr"/>
+      <c r="C13" s="99" t="inlineStr"/>
+      <c r="D13" s="100" t="inlineStr"/>
+      <c r="E13" s="99" t="inlineStr"/>
+      <c r="F13" s="100" t="inlineStr"/>
+      <c r="G13" s="99" t="inlineStr"/>
+      <c r="H13" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I13" s="100" t="inlineStr"/>
+      <c r="J13" s="101">
+        <f>IF(B13="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B13&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K13" s="101">
+        <f>IF(B13="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B13&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L13" s="102">
+        <f>IF(B13="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B13&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M13" s="102">
+        <f>IF(B13="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B13&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N13" s="99" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="103" t="inlineStr">
+        <is>
+          <t>AGT-006</t>
+        </is>
+      </c>
+      <c r="B14" s="104" t="inlineStr"/>
+      <c r="C14" s="105" t="inlineStr"/>
+      <c r="D14" s="106" t="inlineStr"/>
+      <c r="E14" s="105" t="inlineStr"/>
+      <c r="F14" s="106" t="inlineStr"/>
+      <c r="G14" s="105" t="inlineStr"/>
+      <c r="H14" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I14" s="106" t="inlineStr"/>
+      <c r="J14" s="107">
+        <f>IF(B14="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B14&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K14" s="107">
+        <f>IF(B14="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B14&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L14" s="108">
+        <f>IF(B14="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B14&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M14" s="108">
+        <f>IF(B14="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B14&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N14" s="105" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="97" t="inlineStr">
+        <is>
+          <t>AGT-007</t>
+        </is>
+      </c>
+      <c r="B15" s="98" t="inlineStr"/>
+      <c r="C15" s="99" t="inlineStr"/>
+      <c r="D15" s="100" t="inlineStr"/>
+      <c r="E15" s="99" t="inlineStr"/>
+      <c r="F15" s="100" t="inlineStr"/>
+      <c r="G15" s="99" t="inlineStr"/>
+      <c r="H15" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I15" s="100" t="inlineStr"/>
+      <c r="J15" s="101">
+        <f>IF(B15="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B15&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K15" s="101">
+        <f>IF(B15="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B15&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L15" s="102">
+        <f>IF(B15="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B15&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M15" s="102">
+        <f>IF(B15="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B15&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N15" s="99" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="103" t="inlineStr">
+        <is>
+          <t>AGT-008</t>
+        </is>
+      </c>
+      <c r="B16" s="104" t="inlineStr"/>
+      <c r="C16" s="105" t="inlineStr"/>
+      <c r="D16" s="106" t="inlineStr"/>
+      <c r="E16" s="105" t="inlineStr"/>
+      <c r="F16" s="106" t="inlineStr"/>
+      <c r="G16" s="105" t="inlineStr"/>
+      <c r="H16" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I16" s="106" t="inlineStr"/>
+      <c r="J16" s="107">
+        <f>IF(B16="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B16&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K16" s="107">
+        <f>IF(B16="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B16&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L16" s="108">
+        <f>IF(B16="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B16&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M16" s="108">
+        <f>IF(B16="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B16&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N16" s="105" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="97" t="inlineStr">
+        <is>
+          <t>AGT-009</t>
+        </is>
+      </c>
+      <c r="B17" s="98" t="inlineStr"/>
+      <c r="C17" s="99" t="inlineStr"/>
+      <c r="D17" s="100" t="inlineStr"/>
+      <c r="E17" s="99" t="inlineStr"/>
+      <c r="F17" s="100" t="inlineStr"/>
+      <c r="G17" s="99" t="inlineStr"/>
+      <c r="H17" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I17" s="100" t="inlineStr"/>
+      <c r="J17" s="101">
+        <f>IF(B17="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B17&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K17" s="101">
+        <f>IF(B17="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B17&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L17" s="102">
+        <f>IF(B17="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B17&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M17" s="102">
+        <f>IF(B17="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B17&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N17" s="99" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="103" t="inlineStr">
+        <is>
+          <t>AGT-010</t>
+        </is>
+      </c>
+      <c r="B18" s="104" t="inlineStr"/>
+      <c r="C18" s="105" t="inlineStr"/>
+      <c r="D18" s="106" t="inlineStr"/>
+      <c r="E18" s="105" t="inlineStr"/>
+      <c r="F18" s="106" t="inlineStr"/>
+      <c r="G18" s="105" t="inlineStr"/>
+      <c r="H18" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I18" s="106" t="inlineStr"/>
+      <c r="J18" s="107">
+        <f>IF(B18="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B18&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K18" s="107">
+        <f>IF(B18="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B18&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L18" s="108">
+        <f>IF(B18="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B18&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M18" s="108">
+        <f>IF(B18="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B18&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N18" s="105" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="97" t="inlineStr">
+        <is>
+          <t>AGT-011</t>
+        </is>
+      </c>
+      <c r="B19" s="98" t="inlineStr"/>
+      <c r="C19" s="99" t="inlineStr"/>
+      <c r="D19" s="100" t="inlineStr"/>
+      <c r="E19" s="99" t="inlineStr"/>
+      <c r="F19" s="100" t="inlineStr"/>
+      <c r="G19" s="99" t="inlineStr"/>
+      <c r="H19" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I19" s="100" t="inlineStr"/>
+      <c r="J19" s="101">
+        <f>IF(B19="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B19&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K19" s="101">
+        <f>IF(B19="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B19&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L19" s="102">
+        <f>IF(B19="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B19&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M19" s="102">
+        <f>IF(B19="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B19&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N19" s="99" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="103" t="inlineStr">
+        <is>
+          <t>AGT-012</t>
+        </is>
+      </c>
+      <c r="B20" s="104" t="inlineStr"/>
+      <c r="C20" s="105" t="inlineStr"/>
+      <c r="D20" s="106" t="inlineStr"/>
+      <c r="E20" s="105" t="inlineStr"/>
+      <c r="F20" s="106" t="inlineStr"/>
+      <c r="G20" s="105" t="inlineStr"/>
+      <c r="H20" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I20" s="106" t="inlineStr"/>
+      <c r="J20" s="107">
+        <f>IF(B20="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B20&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K20" s="107">
+        <f>IF(B20="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B20&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L20" s="108">
+        <f>IF(B20="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B20&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M20" s="108">
+        <f>IF(B20="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B20&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N20" s="105" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="97" t="inlineStr">
+        <is>
+          <t>AGT-013</t>
+        </is>
+      </c>
+      <c r="B21" s="98" t="inlineStr"/>
+      <c r="C21" s="99" t="inlineStr"/>
+      <c r="D21" s="100" t="inlineStr"/>
+      <c r="E21" s="99" t="inlineStr"/>
+      <c r="F21" s="100" t="inlineStr"/>
+      <c r="G21" s="99" t="inlineStr"/>
+      <c r="H21" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I21" s="100" t="inlineStr"/>
+      <c r="J21" s="101">
+        <f>IF(B21="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B21&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K21" s="101">
+        <f>IF(B21="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B21&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L21" s="102">
+        <f>IF(B21="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B21&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M21" s="102">
+        <f>IF(B21="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B21&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N21" s="99" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="103" t="inlineStr">
+        <is>
+          <t>AGT-014</t>
+        </is>
+      </c>
+      <c r="B22" s="104" t="inlineStr"/>
+      <c r="C22" s="105" t="inlineStr"/>
+      <c r="D22" s="106" t="inlineStr"/>
+      <c r="E22" s="105" t="inlineStr"/>
+      <c r="F22" s="106" t="inlineStr"/>
+      <c r="G22" s="105" t="inlineStr"/>
+      <c r="H22" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I22" s="106" t="inlineStr"/>
+      <c r="J22" s="107">
+        <f>IF(B22="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B22&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K22" s="107">
+        <f>IF(B22="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B22&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L22" s="108">
+        <f>IF(B22="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B22&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M22" s="108">
+        <f>IF(B22="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B22&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N22" s="105" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="97" t="inlineStr">
+        <is>
+          <t>AGT-015</t>
+        </is>
+      </c>
+      <c r="B23" s="98" t="inlineStr"/>
+      <c r="C23" s="99" t="inlineStr"/>
+      <c r="D23" s="100" t="inlineStr"/>
+      <c r="E23" s="99" t="inlineStr"/>
+      <c r="F23" s="100" t="inlineStr"/>
+      <c r="G23" s="99" t="inlineStr"/>
+      <c r="H23" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I23" s="100" t="inlineStr"/>
+      <c r="J23" s="101">
+        <f>IF(B23="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B23&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K23" s="101">
+        <f>IF(B23="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B23&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L23" s="102">
+        <f>IF(B23="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B23&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M23" s="102">
+        <f>IF(B23="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B23&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N23" s="99" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="103" t="inlineStr">
+        <is>
+          <t>AGT-016</t>
+        </is>
+      </c>
+      <c r="B24" s="104" t="inlineStr"/>
+      <c r="C24" s="105" t="inlineStr"/>
+      <c r="D24" s="106" t="inlineStr"/>
+      <c r="E24" s="105" t="inlineStr"/>
+      <c r="F24" s="106" t="inlineStr"/>
+      <c r="G24" s="105" t="inlineStr"/>
+      <c r="H24" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I24" s="106" t="inlineStr"/>
+      <c r="J24" s="107">
+        <f>IF(B24="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B24&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K24" s="107">
+        <f>IF(B24="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B24&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L24" s="108">
+        <f>IF(B24="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B24&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M24" s="108">
+        <f>IF(B24="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B24&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N24" s="105" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="97" t="inlineStr">
+        <is>
+          <t>AGT-017</t>
+        </is>
+      </c>
+      <c r="B25" s="98" t="inlineStr"/>
+      <c r="C25" s="99" t="inlineStr"/>
+      <c r="D25" s="100" t="inlineStr"/>
+      <c r="E25" s="99" t="inlineStr"/>
+      <c r="F25" s="100" t="inlineStr"/>
+      <c r="G25" s="99" t="inlineStr"/>
+      <c r="H25" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I25" s="100" t="inlineStr"/>
+      <c r="J25" s="101">
+        <f>IF(B25="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B25&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K25" s="101">
+        <f>IF(B25="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B25&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L25" s="102">
+        <f>IF(B25="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B25&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M25" s="102">
+        <f>IF(B25="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B25&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N25" s="99" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="103" t="inlineStr">
+        <is>
+          <t>AGT-018</t>
+        </is>
+      </c>
+      <c r="B26" s="104" t="inlineStr"/>
+      <c r="C26" s="105" t="inlineStr"/>
+      <c r="D26" s="106" t="inlineStr"/>
+      <c r="E26" s="105" t="inlineStr"/>
+      <c r="F26" s="106" t="inlineStr"/>
+      <c r="G26" s="105" t="inlineStr"/>
+      <c r="H26" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I26" s="106" t="inlineStr"/>
+      <c r="J26" s="107">
+        <f>IF(B26="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B26&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K26" s="107">
+        <f>IF(B26="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B26&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L26" s="108">
+        <f>IF(B26="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B26&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M26" s="108">
+        <f>IF(B26="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B26&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N26" s="105" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="97" t="inlineStr">
+        <is>
+          <t>AGT-019</t>
+        </is>
+      </c>
+      <c r="B27" s="98" t="inlineStr"/>
+      <c r="C27" s="99" t="inlineStr"/>
+      <c r="D27" s="100" t="inlineStr"/>
+      <c r="E27" s="99" t="inlineStr"/>
+      <c r="F27" s="100" t="inlineStr"/>
+      <c r="G27" s="99" t="inlineStr"/>
+      <c r="H27" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I27" s="100" t="inlineStr"/>
+      <c r="J27" s="101">
+        <f>IF(B27="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B27&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K27" s="101">
+        <f>IF(B27="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B27&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L27" s="102">
+        <f>IF(B27="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B27&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M27" s="102">
+        <f>IF(B27="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B27&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N27" s="99" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="103" t="inlineStr">
+        <is>
+          <t>AGT-020</t>
+        </is>
+      </c>
+      <c r="B28" s="104" t="inlineStr"/>
+      <c r="C28" s="105" t="inlineStr"/>
+      <c r="D28" s="106" t="inlineStr"/>
+      <c r="E28" s="105" t="inlineStr"/>
+      <c r="F28" s="106" t="inlineStr"/>
+      <c r="G28" s="105" t="inlineStr"/>
+      <c r="H28" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I28" s="106" t="inlineStr"/>
+      <c r="J28" s="107">
+        <f>IF(B28="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B28&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K28" s="107">
+        <f>IF(B28="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B28&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L28" s="108">
+        <f>IF(B28="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B28&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M28" s="108">
+        <f>IF(B28="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B28&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N28" s="105" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="97" t="inlineStr">
+        <is>
+          <t>AGT-021</t>
+        </is>
+      </c>
+      <c r="B29" s="98" t="inlineStr"/>
+      <c r="C29" s="99" t="inlineStr"/>
+      <c r="D29" s="100" t="inlineStr"/>
+      <c r="E29" s="99" t="inlineStr"/>
+      <c r="F29" s="100" t="inlineStr"/>
+      <c r="G29" s="99" t="inlineStr"/>
+      <c r="H29" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I29" s="100" t="inlineStr"/>
+      <c r="J29" s="101">
+        <f>IF(B29="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B29&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K29" s="101">
+        <f>IF(B29="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B29&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L29" s="102">
+        <f>IF(B29="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B29&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M29" s="102">
+        <f>IF(B29="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B29&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N29" s="99" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="103" t="inlineStr">
+        <is>
+          <t>AGT-022</t>
+        </is>
+      </c>
+      <c r="B30" s="104" t="inlineStr"/>
+      <c r="C30" s="105" t="inlineStr"/>
+      <c r="D30" s="106" t="inlineStr"/>
+      <c r="E30" s="105" t="inlineStr"/>
+      <c r="F30" s="106" t="inlineStr"/>
+      <c r="G30" s="105" t="inlineStr"/>
+      <c r="H30" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I30" s="106" t="inlineStr"/>
+      <c r="J30" s="107">
+        <f>IF(B30="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B30&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K30" s="107">
+        <f>IF(B30="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B30&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L30" s="108">
+        <f>IF(B30="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B30&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M30" s="108">
+        <f>IF(B30="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B30&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N30" s="105" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="97" t="inlineStr">
+        <is>
+          <t>AGT-023</t>
+        </is>
+      </c>
+      <c r="B31" s="98" t="inlineStr"/>
+      <c r="C31" s="99" t="inlineStr"/>
+      <c r="D31" s="100" t="inlineStr"/>
+      <c r="E31" s="99" t="inlineStr"/>
+      <c r="F31" s="100" t="inlineStr"/>
+      <c r="G31" s="99" t="inlineStr"/>
+      <c r="H31" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I31" s="100" t="inlineStr"/>
+      <c r="J31" s="101">
+        <f>IF(B31="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B31&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K31" s="101">
+        <f>IF(B31="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B31&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L31" s="102">
+        <f>IF(B31="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B31&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M31" s="102">
+        <f>IF(B31="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B31&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N31" s="99" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="103" t="inlineStr">
+        <is>
+          <t>AGT-024</t>
+        </is>
+      </c>
+      <c r="B32" s="104" t="inlineStr"/>
+      <c r="C32" s="105" t="inlineStr"/>
+      <c r="D32" s="106" t="inlineStr"/>
+      <c r="E32" s="105" t="inlineStr"/>
+      <c r="F32" s="106" t="inlineStr"/>
+      <c r="G32" s="105" t="inlineStr"/>
+      <c r="H32" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I32" s="106" t="inlineStr"/>
+      <c r="J32" s="107">
+        <f>IF(B32="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B32&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K32" s="107">
+        <f>IF(B32="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B32&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L32" s="108">
+        <f>IF(B32="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B32&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M32" s="108">
+        <f>IF(B32="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B32&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N32" s="105" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="97" t="inlineStr">
+        <is>
+          <t>AGT-025</t>
+        </is>
+      </c>
+      <c r="B33" s="98" t="inlineStr"/>
+      <c r="C33" s="99" t="inlineStr"/>
+      <c r="D33" s="100" t="inlineStr"/>
+      <c r="E33" s="99" t="inlineStr"/>
+      <c r="F33" s="100" t="inlineStr"/>
+      <c r="G33" s="99" t="inlineStr"/>
+      <c r="H33" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I33" s="100" t="inlineStr"/>
+      <c r="J33" s="101">
+        <f>IF(B33="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B33&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K33" s="101">
+        <f>IF(B33="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B33&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L33" s="102">
+        <f>IF(B33="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B33&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M33" s="102">
+        <f>IF(B33="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B33&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N33" s="99" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="103" t="inlineStr">
+        <is>
+          <t>AGT-026</t>
+        </is>
+      </c>
+      <c r="B34" s="104" t="inlineStr"/>
+      <c r="C34" s="105" t="inlineStr"/>
+      <c r="D34" s="106" t="inlineStr"/>
+      <c r="E34" s="105" t="inlineStr"/>
+      <c r="F34" s="106" t="inlineStr"/>
+      <c r="G34" s="105" t="inlineStr"/>
+      <c r="H34" s="106" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I34" s="106" t="inlineStr"/>
+      <c r="J34" s="107">
+        <f>IF(B34="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B34&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K34" s="107">
+        <f>IF(B34="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B34&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L34" s="108">
+        <f>IF(B34="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B34&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M34" s="108">
+        <f>IF(B34="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B34&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N34" s="105" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="97" t="inlineStr">
+        <is>
+          <t>AGT-027</t>
+        </is>
+      </c>
+      <c r="B35" s="98" t="inlineStr"/>
+      <c r="C35" s="99" t="inlineStr"/>
+      <c r="D35" s="100" t="inlineStr"/>
+      <c r="E35" s="99" t="inlineStr"/>
+      <c r="F35" s="100" t="inlineStr"/>
+      <c r="G35" s="99" t="inlineStr"/>
+      <c r="H35" s="100" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I35" s="100" t="inlineStr"/>
+      <c r="J35" s="101">
+        <f>IF(B35="","",COUNTIF('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B35&amp;"*"))</f>
+        <v/>
+      </c>
+      <c r="K35" s="101">
+        <f>IF(B35="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B35&amp;"*", 'Recruit Monitoring Tracker'!$H$9:$H$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="L35" s="102">
+        <f>IF(B35="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B35&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "In Progress"))</f>
+        <v/>
+      </c>
+      <c r="M35" s="102">
+        <f>IF(B35="","",COUNTIFS('Recruit Monitoring Tracker'!$E$9:$E$65, "*"&amp;B35&amp;"*", 'Recruit Monitoring Tracker'!$L$9:$L$65, "Yes"))</f>
+        <v/>
+      </c>
+      <c r="N35" s="99" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H9:H35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Active,Inactive,On Leave,Pending Verification"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>